<commit_message>
Add new AI judgements to csvs
</commit_message>
<xml_diff>
--- a/data/LVR_screening_sheet_2.xlsx
+++ b/data/LVR_screening_sheet_2.xlsx
@@ -3243,7 +3243,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:P128"/>
+  <dimension ref="A1:Q128"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -3262,9 +3262,10 @@
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="28" customWidth="1"/>
     <col min="16" max="16" width="55" customWidth="1"/>
+    <col min="17" max="17" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:17" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
         <v>29</v>
       </c>
@@ -3313,8 +3314,13 @@
       <c r="P1" s="8" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q1" s="8" t="inlineStr">
+        <is>
+          <t>Re-screen decision (AI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="9">
         <v>1</v>
       </c>
@@ -3353,8 +3359,9 @@
       <c r="P2" s="12" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q2" s="12"/>
+    </row>
+    <row r="3" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="9">
         <v>2</v>
       </c>
@@ -3397,8 +3404,9 @@
       <c r="P3" s="12" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="4" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q3" s="12"/>
+    </row>
+    <row r="4" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="9">
         <v>3</v>
       </c>
@@ -3441,8 +3449,9 @@
       <c r="P4" s="12" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="5" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q4" s="12"/>
+    </row>
+    <row r="5" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="9">
         <v>4</v>
       </c>
@@ -3485,8 +3494,9 @@
       <c r="P5" s="12" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="6" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q5" s="12"/>
+    </row>
+    <row r="6" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="9">
         <v>5</v>
       </c>
@@ -3525,8 +3535,9 @@
       <c r="P6" s="12" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="7" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q6" s="12"/>
+    </row>
+    <row r="7" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="9">
         <v>6</v>
       </c>
@@ -3569,8 +3580,9 @@
       <c r="P7" s="12" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="8" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q7" s="12"/>
+    </row>
+    <row r="8" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9">
         <v>7</v>
       </c>
@@ -3613,8 +3625,9 @@
       <c r="P8" s="12" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="9" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q8" s="12"/>
+    </row>
+    <row r="9" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="9">
         <v>8</v>
       </c>
@@ -3657,8 +3670,9 @@
       <c r="P9" s="12" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="10" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q9" s="12"/>
+    </row>
+    <row r="10" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="9">
         <v>9</v>
       </c>
@@ -3701,8 +3715,9 @@
       <c r="P10" s="12" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="11" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q10" s="12"/>
+    </row>
+    <row r="11" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="9">
         <v>10</v>
       </c>
@@ -3745,8 +3760,9 @@
       <c r="P11" s="12" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="12" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q11" s="12"/>
+    </row>
+    <row r="12" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="9">
         <v>11</v>
       </c>
@@ -3789,8 +3805,9 @@
       <c r="P12" s="12" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="13" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q12" s="12"/>
+    </row>
+    <row r="13" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="9">
         <v>12</v>
       </c>
@@ -3831,8 +3848,9 @@
       <c r="P13" s="12" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="14" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q13" s="12"/>
+    </row>
+    <row r="14" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="9">
         <v>13</v>
       </c>
@@ -3875,8 +3893,9 @@
       <c r="P14" s="12" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="15" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q14" s="12"/>
+    </row>
+    <row r="15" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="9">
         <v>14</v>
       </c>
@@ -3917,8 +3936,9 @@
       <c r="P15" s="12" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="16" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q15" s="12"/>
+    </row>
+    <row r="16" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="9">
         <v>15</v>
       </c>
@@ -3961,8 +3981,9 @@
       <c r="P16" s="12" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="17" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q16" s="12"/>
+    </row>
+    <row r="17" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="9">
         <v>16</v>
       </c>
@@ -4003,8 +4024,9 @@
       <c r="P17" s="12" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="18" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q17" s="12"/>
+    </row>
+    <row r="18" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="9">
         <v>17</v>
       </c>
@@ -4047,8 +4069,9 @@
       <c r="P18" s="12" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="19" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q18" s="12"/>
+    </row>
+    <row r="19" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="9">
         <v>18</v>
       </c>
@@ -4089,8 +4112,9 @@
       <c r="P19" s="12" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="20" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q19" s="12"/>
+    </row>
+    <row r="20" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="9">
         <v>19</v>
       </c>
@@ -4133,8 +4157,9 @@
       <c r="P20" s="12" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="21" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q20" s="12"/>
+    </row>
+    <row r="21" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="9">
         <v>20</v>
       </c>
@@ -4175,8 +4200,9 @@
       <c r="P21" s="12" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="22" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q21" s="12"/>
+    </row>
+    <row r="22" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="9">
         <v>21</v>
       </c>
@@ -4217,8 +4243,9 @@
       <c r="P22" s="12" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="23" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q22" s="12"/>
+    </row>
+    <row r="23" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="9">
         <v>22</v>
       </c>
@@ -4261,8 +4288,9 @@
       <c r="P23" s="12" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="24" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q23" s="12"/>
+    </row>
+    <row r="24" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="9">
         <v>23</v>
       </c>
@@ -4303,8 +4331,9 @@
       <c r="P24" s="12" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="25" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q24" s="12"/>
+    </row>
+    <row r="25" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="9">
         <v>24</v>
       </c>
@@ -4347,8 +4376,9 @@
       <c r="P25" s="12" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="26" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q25" s="12"/>
+    </row>
+    <row r="26" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="9">
         <v>25</v>
       </c>
@@ -4391,8 +4421,9 @@
       <c r="P26" s="12" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="27" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q26" s="12"/>
+    </row>
+    <row r="27" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="9">
         <v>26</v>
       </c>
@@ -4431,8 +4462,9 @@
       <c r="P27" s="12" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="28" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q27" s="12"/>
+    </row>
+    <row r="28" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="9">
         <v>27</v>
       </c>
@@ -4471,8 +4503,9 @@
       <c r="P28" s="12" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="29" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q28" s="12"/>
+    </row>
+    <row r="29" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="9">
         <v>28</v>
       </c>
@@ -4515,8 +4548,9 @@
       <c r="P29" s="12" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="30" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q29" s="12"/>
+    </row>
+    <row r="30" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="9">
         <v>29</v>
       </c>
@@ -4557,8 +4591,9 @@
       <c r="P30" s="12" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="31" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q30" s="12"/>
+    </row>
+    <row r="31" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="9">
         <v>30</v>
       </c>
@@ -4597,8 +4632,9 @@
       <c r="P31" s="12" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="32" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q31" s="12"/>
+    </row>
+    <row r="32" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="9">
         <v>31</v>
       </c>
@@ -4639,8 +4675,9 @@
       <c r="P32" s="12" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="33" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q32" s="12"/>
+    </row>
+    <row r="33" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="9">
         <v>32</v>
       </c>
@@ -4683,8 +4720,9 @@
       <c r="P33" s="12" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="34" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q33" s="12"/>
+    </row>
+    <row r="34" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="9">
         <v>33</v>
       </c>
@@ -4727,8 +4765,9 @@
       <c r="P34" s="12" t="s">
         <v>241</v>
       </c>
-    </row>
-    <row r="35" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q34" s="12"/>
+    </row>
+    <row r="35" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="9">
         <v>34</v>
       </c>
@@ -4769,8 +4808,9 @@
       <c r="P35" s="12" t="s">
         <v>247</v>
       </c>
-    </row>
-    <row r="36" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q35" s="12"/>
+    </row>
+    <row r="36" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="9">
         <v>35</v>
       </c>
@@ -4813,8 +4853,9 @@
       <c r="P36" s="12" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="37" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q36" s="12"/>
+    </row>
+    <row r="37" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="9">
         <v>36</v>
       </c>
@@ -4855,8 +4896,9 @@
       <c r="P37" s="12" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="38" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q37" s="12"/>
+    </row>
+    <row r="38" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="9">
         <v>37</v>
       </c>
@@ -4895,8 +4937,9 @@
       <c r="P38" s="12" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="39" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q38" s="12"/>
+    </row>
+    <row r="39" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="9">
         <v>38</v>
       </c>
@@ -4935,8 +4978,9 @@
       <c r="P39" s="12" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="40" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q39" s="12"/>
+    </row>
+    <row r="40" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="9">
         <v>39</v>
       </c>
@@ -4975,8 +5019,9 @@
       <c r="P40" s="12" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="41" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q40" s="12"/>
+    </row>
+    <row r="41" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="9">
         <v>40</v>
       </c>
@@ -5019,8 +5064,9 @@
       <c r="P41" s="12" t="s">
         <v>283</v>
       </c>
-    </row>
-    <row r="42" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q41" s="12"/>
+    </row>
+    <row r="42" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="9">
         <v>41</v>
       </c>
@@ -5057,8 +5103,13 @@
       <c r="P42" s="12" t="s">
         <v>289</v>
       </c>
-    </row>
-    <row r="43" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q42" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="9">
         <v>42</v>
       </c>
@@ -5097,8 +5148,13 @@
       <c r="P43" s="12" t="s">
         <v>295</v>
       </c>
-    </row>
-    <row r="44" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q43" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="9">
         <v>43</v>
       </c>
@@ -5137,8 +5193,13 @@
       <c r="P44" s="12" t="s">
         <v>301</v>
       </c>
-    </row>
-    <row r="45" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q44" s="12" t="inlineStr">
+        <is>
+          <t>Maybe</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="9">
         <v>44</v>
       </c>
@@ -5177,8 +5238,13 @@
       <c r="P45" s="12" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="46" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q45" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="9">
         <v>45</v>
       </c>
@@ -5217,8 +5283,13 @@
       <c r="P46" s="12" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="47" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q46" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="9">
         <v>46</v>
       </c>
@@ -5255,8 +5326,13 @@
       <c r="P47" s="12" t="s">
         <v>317</v>
       </c>
-    </row>
-    <row r="48" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q47" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="9">
         <v>47</v>
       </c>
@@ -5293,8 +5369,13 @@
       <c r="P48" s="12" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="49" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q48" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="9">
         <v>48</v>
       </c>
@@ -5331,8 +5412,13 @@
       <c r="P49" s="12" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="50" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q49" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="9">
         <v>49</v>
       </c>
@@ -5371,8 +5457,13 @@
       <c r="P50" s="12" t="s">
         <v>333</v>
       </c>
-    </row>
-    <row r="51" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q50" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="9">
         <v>50</v>
       </c>
@@ -5411,8 +5502,13 @@
       <c r="P51" s="12" t="s">
         <v>339</v>
       </c>
-    </row>
-    <row r="52" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q51" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="9">
         <v>51</v>
       </c>
@@ -5451,8 +5547,13 @@
       <c r="P52" s="12" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="53" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q52" s="12" t="inlineStr">
+        <is>
+          <t>Maybe</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="9">
         <v>52</v>
       </c>
@@ -5491,8 +5592,13 @@
       <c r="P53" s="12" t="s">
         <v>351</v>
       </c>
-    </row>
-    <row r="54" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q53" s="12" t="inlineStr">
+        <is>
+          <t>Maybe</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="9">
         <v>53</v>
       </c>
@@ -5531,8 +5637,13 @@
       <c r="P54" s="12" t="s">
         <v>357</v>
       </c>
-    </row>
-    <row r="55" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q54" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="9">
         <v>54</v>
       </c>
@@ -5571,8 +5682,13 @@
       <c r="P55" s="12" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="56" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q55" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="9">
         <v>55</v>
       </c>
@@ -5609,8 +5725,13 @@
       <c r="P56" s="12" t="s">
         <v>368</v>
       </c>
-    </row>
-    <row r="57" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q56" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="9">
         <v>56</v>
       </c>
@@ -5649,8 +5770,13 @@
       <c r="P57" s="12" t="s">
         <v>374</v>
       </c>
-    </row>
-    <row r="58" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q57" s="12" t="inlineStr">
+        <is>
+          <t>Maybe</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="9">
         <v>57</v>
       </c>
@@ -5689,8 +5815,13 @@
       <c r="P58" s="12" t="s">
         <v>380</v>
       </c>
-    </row>
-    <row r="59" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q58" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="9">
         <v>58</v>
       </c>
@@ -5729,8 +5860,13 @@
       <c r="P59" s="12" t="s">
         <v>385</v>
       </c>
-    </row>
-    <row r="60" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q59" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="9">
         <v>59</v>
       </c>
@@ -5769,8 +5905,13 @@
       <c r="P60" s="12" t="s">
         <v>391</v>
       </c>
-    </row>
-    <row r="61" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q60" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="9">
         <v>60</v>
       </c>
@@ -5809,8 +5950,13 @@
       <c r="P61" s="12" t="s">
         <v>396</v>
       </c>
-    </row>
-    <row r="62" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q61" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="9">
         <v>61</v>
       </c>
@@ -5849,8 +5995,13 @@
       <c r="P62" s="12" t="s">
         <v>402</v>
       </c>
-    </row>
-    <row r="63" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q62" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="9">
         <v>62</v>
       </c>
@@ -5889,8 +6040,13 @@
       <c r="P63" s="12" t="s">
         <v>408</v>
       </c>
-    </row>
-    <row r="64" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q63" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="9">
         <v>63</v>
       </c>
@@ -5927,8 +6083,13 @@
       <c r="P64" s="12" t="s">
         <v>414</v>
       </c>
-    </row>
-    <row r="65" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q64" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="9">
         <v>64</v>
       </c>
@@ -5967,8 +6128,13 @@
       <c r="P65" s="12" t="s">
         <v>420</v>
       </c>
-    </row>
-    <row r="66" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q65" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="9">
         <v>65</v>
       </c>
@@ -6005,8 +6171,13 @@
       <c r="P66" s="12" t="s">
         <v>425</v>
       </c>
-    </row>
-    <row r="67" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q66" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="9">
         <v>66</v>
       </c>
@@ -6043,8 +6214,13 @@
       <c r="P67" s="12" t="s">
         <v>429</v>
       </c>
-    </row>
-    <row r="68" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q67" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="9">
         <v>67</v>
       </c>
@@ -6081,8 +6257,13 @@
       <c r="P68" s="12" t="s">
         <v>435</v>
       </c>
-    </row>
-    <row r="69" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q68" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="9">
         <v>68</v>
       </c>
@@ -6121,8 +6302,13 @@
       <c r="P69" s="12" t="s">
         <v>441</v>
       </c>
-    </row>
-    <row r="70" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q69" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="9">
         <v>69</v>
       </c>
@@ -6161,8 +6347,13 @@
       <c r="P70" s="12" t="s">
         <v>446</v>
       </c>
-    </row>
-    <row r="71" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q70" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="9">
         <v>70</v>
       </c>
@@ -6201,8 +6392,13 @@
       <c r="P71" s="12" t="s">
         <v>451</v>
       </c>
-    </row>
-    <row r="72" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q71" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="9">
         <v>71</v>
       </c>
@@ -6241,8 +6437,13 @@
       <c r="P72" s="12" t="s">
         <v>457</v>
       </c>
-    </row>
-    <row r="73" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q72" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="9">
         <v>72</v>
       </c>
@@ -6279,8 +6480,13 @@
       <c r="P73" s="12" t="s">
         <v>462</v>
       </c>
-    </row>
-    <row r="74" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q73" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="9">
         <v>73</v>
       </c>
@@ -6317,8 +6523,13 @@
       <c r="P74" s="12" t="s">
         <v>467</v>
       </c>
-    </row>
-    <row r="75" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q74" s="12" t="inlineStr">
+        <is>
+          <t>Maybe</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="9">
         <v>74</v>
       </c>
@@ -6355,8 +6566,13 @@
       <c r="P75" s="12" t="s">
         <v>473</v>
       </c>
-    </row>
-    <row r="76" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q75" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="9">
         <v>75</v>
       </c>
@@ -6395,8 +6611,13 @@
       <c r="P76" s="12" t="s">
         <v>479</v>
       </c>
-    </row>
-    <row r="77" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q76" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="9">
         <v>76</v>
       </c>
@@ -6435,8 +6656,13 @@
       <c r="P77" s="12" t="s">
         <v>484</v>
       </c>
-    </row>
-    <row r="78" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q77" s="12" t="inlineStr">
+        <is>
+          <t>Maybe</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="9">
         <v>77</v>
       </c>
@@ -6475,8 +6701,13 @@
       <c r="P78" s="12" t="s">
         <v>490</v>
       </c>
-    </row>
-    <row r="79" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q78" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="9">
         <v>78</v>
       </c>
@@ -6515,8 +6746,13 @@
       <c r="P79" s="12" t="s">
         <v>496</v>
       </c>
-    </row>
-    <row r="80" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q79" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="9">
         <v>79</v>
       </c>
@@ -6553,8 +6789,13 @@
       <c r="P80" s="12" t="s">
         <v>502</v>
       </c>
-    </row>
-    <row r="81" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q80" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="9">
         <v>80</v>
       </c>
@@ -6593,8 +6834,13 @@
       <c r="P81" s="12" t="s">
         <v>507</v>
       </c>
-    </row>
-    <row r="82" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q81" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="9">
         <v>81</v>
       </c>
@@ -6633,8 +6879,13 @@
       <c r="P82" s="12" t="s">
         <v>513</v>
       </c>
-    </row>
-    <row r="83" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q82" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="9">
         <v>82</v>
       </c>
@@ -6673,8 +6924,13 @@
       <c r="P83" s="12" t="s">
         <v>519</v>
       </c>
-    </row>
-    <row r="84" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q83" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="9">
         <v>83</v>
       </c>
@@ -6713,8 +6969,13 @@
       <c r="P84" s="12" t="s">
         <v>525</v>
       </c>
-    </row>
-    <row r="85" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q84" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="9">
         <v>84</v>
       </c>
@@ -6751,8 +7012,13 @@
       <c r="P85" s="12" t="s">
         <v>531</v>
       </c>
-    </row>
-    <row r="86" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q85" s="12" t="inlineStr">
+        <is>
+          <t>Maybe</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="9">
         <v>85</v>
       </c>
@@ -6791,8 +7057,13 @@
       <c r="P86" s="12" t="s">
         <v>537</v>
       </c>
-    </row>
-    <row r="87" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q86" s="12" t="inlineStr">
+        <is>
+          <t>Maybe</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="9">
         <v>86</v>
       </c>
@@ -6829,8 +7100,13 @@
       <c r="P87" s="12" t="s">
         <v>542</v>
       </c>
-    </row>
-    <row r="88" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q87" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="9">
         <v>87</v>
       </c>
@@ -6869,8 +7145,13 @@
       <c r="P88" s="12" t="s">
         <v>548</v>
       </c>
-    </row>
-    <row r="89" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q88" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="9">
         <v>88</v>
       </c>
@@ -6909,8 +7190,13 @@
       <c r="P89" s="12" t="s">
         <v>553</v>
       </c>
-    </row>
-    <row r="90" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q89" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="9">
         <v>89</v>
       </c>
@@ -6947,8 +7233,13 @@
       <c r="P90" s="12" t="s">
         <v>559</v>
       </c>
-    </row>
-    <row r="91" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q90" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="9">
         <v>90</v>
       </c>
@@ -6987,8 +7278,13 @@
       <c r="P91" s="12" t="s">
         <v>564</v>
       </c>
-    </row>
-    <row r="92" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q91" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="9">
         <v>91</v>
       </c>
@@ -7027,8 +7323,13 @@
       <c r="P92" s="12" t="s">
         <v>570</v>
       </c>
-    </row>
-    <row r="93" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q92" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="9">
         <v>92</v>
       </c>
@@ -7065,8 +7366,13 @@
       <c r="P93" s="12" t="s">
         <v>575</v>
       </c>
-    </row>
-    <row r="94" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q93" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="9">
         <v>93</v>
       </c>
@@ -7101,8 +7407,13 @@
       <c r="P94" s="12" t="s">
         <v>580</v>
       </c>
-    </row>
-    <row r="95" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q94" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="9">
         <v>94</v>
       </c>
@@ -7141,8 +7452,13 @@
       <c r="P95" s="12" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="96" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q95" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="9">
         <v>95</v>
       </c>
@@ -7181,8 +7497,13 @@
       <c r="P96" s="12" t="s">
         <v>591</v>
       </c>
-    </row>
-    <row r="97" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q96" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="9">
         <v>96</v>
       </c>
@@ -7221,8 +7542,13 @@
       <c r="P97" s="12" t="s">
         <v>597</v>
       </c>
-    </row>
-    <row r="98" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q97" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="9">
         <v>97</v>
       </c>
@@ -7261,8 +7587,13 @@
       <c r="P98" s="12" t="s">
         <v>602</v>
       </c>
-    </row>
-    <row r="99" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q98" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="9">
         <v>98</v>
       </c>
@@ -7301,8 +7632,13 @@
       <c r="P99" s="12" t="s">
         <v>608</v>
       </c>
-    </row>
-    <row r="100" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q99" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="9">
         <v>99</v>
       </c>
@@ -7341,8 +7677,13 @@
       <c r="P100" s="12" t="s">
         <v>613</v>
       </c>
-    </row>
-    <row r="101" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q100" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="9">
         <v>100</v>
       </c>
@@ -7381,8 +7722,13 @@
       <c r="P101" s="12" t="s">
         <v>619</v>
       </c>
-    </row>
-    <row r="102" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q101" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="9">
         <v>101</v>
       </c>
@@ -7421,8 +7767,13 @@
       <c r="P102" s="12" t="s">
         <v>624</v>
       </c>
-    </row>
-    <row r="103" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q102" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="9">
         <v>102</v>
       </c>
@@ -7461,8 +7812,13 @@
       <c r="P103" s="12" t="s">
         <v>630</v>
       </c>
-    </row>
-    <row r="104" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q103" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="9">
         <v>103</v>
       </c>
@@ -7501,8 +7857,13 @@
       <c r="P104" s="12" t="s">
         <v>635</v>
       </c>
-    </row>
-    <row r="105" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q104" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="9">
         <v>104</v>
       </c>
@@ -7541,8 +7902,13 @@
       <c r="P105" s="12" t="s">
         <v>641</v>
       </c>
-    </row>
-    <row r="106" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q105" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="9">
         <v>105</v>
       </c>
@@ -7579,8 +7945,13 @@
       <c r="P106" s="12" t="s">
         <v>647</v>
       </c>
-    </row>
-    <row r="107" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q106" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="9">
         <v>106</v>
       </c>
@@ -7619,8 +7990,13 @@
       <c r="P107" s="12" t="s">
         <v>652</v>
       </c>
-    </row>
-    <row r="108" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q107" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="9">
         <v>107</v>
       </c>
@@ -7659,8 +8035,13 @@
       <c r="P108" s="12" t="s">
         <v>657</v>
       </c>
-    </row>
-    <row r="109" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q108" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="9">
         <v>108</v>
       </c>
@@ -7697,8 +8078,13 @@
       <c r="P109" s="12" t="s">
         <v>662</v>
       </c>
-    </row>
-    <row r="110" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q109" s="12" t="inlineStr">
+        <is>
+          <t>Maybe</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="9">
         <v>109</v>
       </c>
@@ -7737,8 +8123,13 @@
       <c r="P110" s="12" t="s">
         <v>668</v>
       </c>
-    </row>
-    <row r="111" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q110" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="9">
         <v>110</v>
       </c>
@@ -7775,8 +8166,13 @@
       <c r="P111" s="12" t="s">
         <v>673</v>
       </c>
-    </row>
-    <row r="112" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q111" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="9">
         <v>111</v>
       </c>
@@ -7815,8 +8211,13 @@
       <c r="P112" s="12" t="s">
         <v>679</v>
       </c>
-    </row>
-    <row r="113" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q112" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="9">
         <v>112</v>
       </c>
@@ -7853,8 +8254,13 @@
       <c r="P113" s="12" t="s">
         <v>685</v>
       </c>
-    </row>
-    <row r="114" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q113" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="9">
         <v>113</v>
       </c>
@@ -7893,8 +8299,13 @@
       <c r="P114" s="12" t="s">
         <v>690</v>
       </c>
-    </row>
-    <row r="115" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q114" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="9">
         <v>114</v>
       </c>
@@ -7933,8 +8344,13 @@
       <c r="P115" s="12" t="s">
         <v>697</v>
       </c>
-    </row>
-    <row r="116" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q115" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="9">
         <v>115</v>
       </c>
@@ -7973,8 +8389,13 @@
       <c r="P116" s="12" t="s">
         <v>703</v>
       </c>
-    </row>
-    <row r="117" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q116" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="9">
         <v>116</v>
       </c>
@@ -8013,8 +8434,13 @@
       <c r="P117" s="12" t="s">
         <v>709</v>
       </c>
-    </row>
-    <row r="118" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q117" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="9">
         <v>117</v>
       </c>
@@ -8051,8 +8477,13 @@
       <c r="P118" s="12" t="s">
         <v>714</v>
       </c>
-    </row>
-    <row r="119" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q118" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="9">
         <v>118</v>
       </c>
@@ -8091,8 +8522,13 @@
       <c r="P119" s="12" t="s">
         <v>719</v>
       </c>
-    </row>
-    <row r="120" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q119" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="9">
         <v>119</v>
       </c>
@@ -8129,8 +8565,13 @@
       <c r="P120" s="12" t="s">
         <v>725</v>
       </c>
-    </row>
-    <row r="121" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q120" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="9">
         <v>120</v>
       </c>
@@ -8167,8 +8608,13 @@
       <c r="P121" s="12" t="s">
         <v>731</v>
       </c>
-    </row>
-    <row r="122" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q121" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="9">
         <v>121</v>
       </c>
@@ -8205,8 +8651,13 @@
       <c r="P122" s="12" t="s">
         <v>737</v>
       </c>
-    </row>
-    <row r="123" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q122" s="12" t="inlineStr">
+        <is>
+          <t>Maybe</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="9">
         <v>122</v>
       </c>
@@ -8243,8 +8694,13 @@
       <c r="P123" s="12" t="s">
         <v>743</v>
       </c>
-    </row>
-    <row r="124" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q123" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="9">
         <v>123</v>
       </c>
@@ -8283,8 +8739,13 @@
       <c r="P124" s="12" t="s">
         <v>748</v>
       </c>
-    </row>
-    <row r="125" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q124" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="9">
         <v>124</v>
       </c>
@@ -8323,8 +8784,13 @@
       <c r="P125" s="12" t="s">
         <v>753</v>
       </c>
-    </row>
-    <row r="126" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q125" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="9">
         <v>125</v>
       </c>
@@ -8363,8 +8829,13 @@
       <c r="P126" s="12" t="s">
         <v>759</v>
       </c>
-    </row>
-    <row r="127" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q126" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="9">
         <v>126</v>
       </c>
@@ -8403,8 +8874,13 @@
       <c r="P127" s="12" t="s">
         <v>764</v>
       </c>
-    </row>
-    <row r="128" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q127" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="9">
         <v>127</v>
       </c>
@@ -8443,9 +8919,14 @@
       <c r="P128" s="12" t="s">
         <v>770</v>
       </c>
+      <c r="Q128" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P128" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:Q128" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <conditionalFormatting sqref="H2:H128">
     <cfRule type="expression" dxfId="8" priority="2">
       <formula>H2="Include"</formula>
@@ -8477,6 +8958,17 @@
     </cfRule>
     <cfRule type="expression" dxfId="0" priority="10">
       <formula>N2="Maybe"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q2:Q128">
+    <cfRule type="expression" dxfId="2" priority="11">
+      <formula>Q2="Include"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="12">
+      <formula>Q2="Exclude"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="13">
+      <formula>Q2="Maybe"</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>

</xml_diff>

<commit_message>
Update screening sheets with new AI selections
</commit_message>
<xml_diff>
--- a/data/LVR_screening_sheet_2.xlsx
+++ b/data/LVR_screening_sheet_2.xlsx
@@ -3243,7 +3243,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Q128"/>
+  <dimension ref="A1:R128"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -3263,9 +3263,10 @@
     <col min="15" max="15" width="28" customWidth="1"/>
     <col min="16" max="16" width="55" customWidth="1"/>
     <col min="17" max="17" width="16" customWidth="1"/>
+    <col min="18" max="18" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
         <v>29</v>
       </c>
@@ -3316,11 +3317,16 @@
       </c>
       <c r="Q1" s="8" t="inlineStr">
         <is>
-          <t>Re-screen decision (AI)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Independent T/A decision (AI)</t>
+        </is>
+      </c>
+      <c r="R1" s="8" t="inlineStr">
+        <is>
+          <t>Independent rationale (AI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="9">
         <v>1</v>
       </c>
@@ -3359,9 +3365,18 @@
       <c r="P2" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="Q2" s="12"/>
-    </row>
-    <row r="3" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q2" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R2" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Wrong population (not adults). Study of social support for high school students with visual impairment; children only and no self-report vision instrument evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="9">
         <v>2</v>
       </c>
@@ -3404,9 +3419,18 @@
       <c r="P3" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="Q3" s="12"/>
-    </row>
-    <row r="4" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q3" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R3" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Other (see notes). Case series of 2 patients fitted with multifocal RGP lenses; VFQ-25 used only as an outcome. Case series are excluded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="9">
         <v>3</v>
       </c>
@@ -3449,9 +3473,18 @@
       <c r="P4" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="Q4" s="12"/>
-    </row>
-    <row r="5" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q4" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R4" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No accuracy/validation data. Cross-sectional study of factors linked to adjustment to vision loss; AS-WAS and self-reported activity limitation are used as outcome/predictors, not evaluated as instruments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="9">
         <v>4</v>
       </c>
@@ -3494,9 +3527,18 @@
       <c r="P5" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="Q5" s="12"/>
-    </row>
-    <row r="6" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q5" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R5" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Review/opinion/editorial. Narrative overview of preferred retinal locus and biofeedback training; no questionnaire evaluation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="9">
         <v>5</v>
       </c>
@@ -3535,9 +3577,18 @@
       <c r="P6" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="Q6" s="12"/>
-    </row>
-    <row r="7" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q6" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="R6" s="12" t="inlineStr">
+        <is>
+          <t>Rasch analysis of the APEDS-VFQ visual function questionnaire in 351 visually impaired adults; psychometric validation of a self-report vision instrument.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="9">
         <v>6</v>
       </c>
@@ -3580,9 +3631,18 @@
       <c r="P7" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="Q7" s="12"/>
-    </row>
-    <row r="8" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q7" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R7" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No accuracy/validation data. Nursing-home teleophthalmology study; the NHVQoL questionnaire is administered descriptively, with no accuracy or psychometric evaluation of it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9">
         <v>7</v>
       </c>
@@ -3625,9 +3685,18 @@
       <c r="P8" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="Q8" s="12"/>
-    </row>
-    <row r="9" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q8" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R8" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No questionnaire/screening item. Survey of teachers on assistive technology for blind and low-vision students; no self-report vision instrument is evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="9">
         <v>8</v>
       </c>
@@ -3670,9 +3739,18 @@
       <c r="P9" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="Q9" s="12"/>
-    </row>
-    <row r="10" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q9" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R9" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No questionnaire/screening item. UK Biobank cohort linking measured visual acuity to incident Parkinson's disease; no self-report vision instrument.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="9">
         <v>9</v>
       </c>
@@ -3715,9 +3793,18 @@
       <c r="P10" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="Q10" s="12"/>
-    </row>
-    <row r="11" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q10" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R10" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No questionnaire/screening item. NHATS analysis of measured VI (acuity, contrast) and homebound status; no self-report vision instrument is evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="9">
         <v>10</v>
       </c>
@@ -3760,9 +3847,18 @@
       <c r="P11" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="Q11" s="12"/>
-    </row>
-    <row r="12" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q11" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R11" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No accuracy/validation data. Epidemiological study of diet, mold exposure and VI in older Chinese adults; the VI assessment is only an outcome and is not itself evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="9">
         <v>11</v>
       </c>
@@ -3805,9 +3901,18 @@
       <c r="P12" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="Q12" s="12"/>
-    </row>
-    <row r="13" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q12" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R12" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Not about low vision/visual function. Usability questionnaire for an e-learning course and colour-contrast check; the self-report is about learning preferences, not vision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="9">
         <v>12</v>
       </c>
@@ -3848,9 +3953,18 @@
       <c r="P13" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="Q13" s="12"/>
-    </row>
-    <row r="14" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q13" s="12" t="inlineStr">
+        <is>
+          <t>Maybe</t>
+        </is>
+      </c>
+      <c r="R13" s="12" t="inlineStr">
+        <is>
+          <t>LVROS baseline of 764 LVR patients; reports that VA correlates poorly with self-reported vision quality, relevant to LVR referral. Unclear if any instrument is formally evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="9">
         <v>13</v>
       </c>
@@ -3893,9 +4007,18 @@
       <c r="P14" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="Q14" s="12"/>
-    </row>
-    <row r="15" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q14" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R14" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Intervention study only. Evaluation of a head-mounted electronic low vision aid; the questionnaire only records willingness to use the device.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="9">
         <v>14</v>
       </c>
@@ -3936,9 +4059,18 @@
       <c r="P15" s="12" t="s">
         <v>132</v>
       </c>
-      <c r="Q15" s="12"/>
-    </row>
-    <row r="16" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q15" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R15" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Intervention study only. Pilot study of VEP biofeedback rehabilitation in AMD; VFQ-25 used only as an outcome measure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="9">
         <v>15</v>
       </c>
@@ -3981,9 +4113,18 @@
       <c r="P16" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="Q16" s="12"/>
-    </row>
-    <row r="17" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q16" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R16" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Wrong population (not adults). Review of paediatric assessment of cerebral visual impairment; children only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="9">
         <v>16</v>
       </c>
@@ -4024,9 +4165,18 @@
       <c r="P17" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="Q17" s="12"/>
-    </row>
-    <row r="18" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q17" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R17" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No accuracy/validation data. Chart review of glaucoma patients attending vision rehab; self-reported ADL difficulty only described alongside BCVA/VF/CS, intake instrument not evaluated. Useful background on glaucoma LVR referral.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="9">
         <v>17</v>
       </c>
@@ -4069,9 +4219,18 @@
       <c r="P18" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="Q18" s="12"/>
-    </row>
-    <row r="19" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q18" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R18" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Intervention study only. Outcomes of mobile-clinic LVR measured with the Activity Inventory; MCID used to judge treatment effect, not to evaluate the instrument.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="9">
         <v>18</v>
       </c>
@@ -4112,9 +4271,18 @@
       <c r="P19" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="Q19" s="12"/>
-    </row>
-    <row r="20" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q19" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R19" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Intervention study only. LVROS outcomes of usual LVR care measured with the Activity Inventory; MCID used to quantify rehab effect, not measurement properties.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="9">
         <v>19</v>
       </c>
@@ -4157,9 +4325,18 @@
       <c r="P20" s="12" t="s">
         <v>161</v>
       </c>
-      <c r="Q20" s="12"/>
-    </row>
-    <row r="21" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q20" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R20" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No accuracy/validation data. Path analysis of cognitive appraisals, distress and self-reported disability in LVR patients; questionnaires used as predictors/outcomes, not evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="9">
         <v>20</v>
       </c>
@@ -4200,9 +4377,18 @@
       <c r="P21" s="12" t="s">
         <v>167</v>
       </c>
-      <c r="Q21" s="12"/>
-    </row>
-    <row r="22" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q21" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R21" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Review/opinion/editorial. Narrative review of low vision examination and rehabilitation stages; no original questionnaire data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="9">
         <v>21</v>
       </c>
@@ -4243,9 +4429,18 @@
       <c r="P22" s="12" t="s">
         <v>173</v>
       </c>
-      <c r="Q22" s="12"/>
-    </row>
-    <row r="23" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q22" s="12" t="inlineStr">
+        <is>
+          <t>Maybe</t>
+        </is>
+      </c>
+      <c r="R22" s="12" t="inlineStr">
+        <is>
+          <t>Cochrane review of RCTs in which self-reported vision questions were the community screening tool; reports the effect of such screening on vision (not accuracy), relevant to clinical use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="9">
         <v>22</v>
       </c>
@@ -4288,9 +4483,18 @@
       <c r="P23" s="12" t="s">
         <v>179</v>
       </c>
-      <c r="Q23" s="12"/>
-    </row>
-    <row r="24" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q23" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R23" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No questionnaire/screening item. Compares short visual acuity charts against clinic VA in older adults; performance tests only, no self-report instrument.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="9">
         <v>23</v>
       </c>
@@ -4331,9 +4535,18 @@
       <c r="P24" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="Q24" s="12"/>
-    </row>
-    <row r="25" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q24" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="R24" s="12" t="inlineStr">
+        <is>
+          <t>NHATS older adults: self-reported visual difficulty evaluated against measured VA and contrast sensitivity with AUC, sensitivity and specificity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="9">
         <v>24</v>
       </c>
@@ -4376,9 +4589,18 @@
       <c r="P25" s="12" t="s">
         <v>190</v>
       </c>
-      <c r="Q25" s="12"/>
-    </row>
-    <row r="26" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q25" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R25" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Intervention study only. RCT protocol on cost-effectiveness of basic vision rehabilitation; Activity Inventory used only as primary outcome.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="9">
         <v>25</v>
       </c>
@@ -4421,9 +4643,18 @@
       <c r="P26" s="12" t="s">
         <v>196</v>
       </c>
-      <c r="Q26" s="12"/>
-    </row>
-    <row r="27" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q26" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R26" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Not about low vision/visual function. PHQ-2 depression screening acceptability in LVR/eye-care clients; the screened construct is depression, not vision or LVR need.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="9">
         <v>26</v>
       </c>
@@ -4462,9 +4693,18 @@
       <c r="P27" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="Q27" s="12"/>
-    </row>
-    <row r="28" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q27" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="R27" s="12" t="inlineStr">
+        <is>
+          <t>Development and psychometric validation (internal consistency, reliability, known-groups, responsiveness) of the LVQOL in low vision patients.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="9">
         <v>27</v>
       </c>
@@ -4503,9 +4743,18 @@
       <c r="P28" s="12" t="s">
         <v>207</v>
       </c>
-      <c r="Q28" s="12"/>
-    </row>
-    <row r="29" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q28" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="R28" s="12" t="inlineStr">
+        <is>
+          <t>Validates Visual Impairment as a Risk for Falls Questionnaire items (e.g. reading, faces) against oculo-visual exam, with sensitivity and specificity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="9">
         <v>28</v>
       </c>
@@ -4548,9 +4797,18 @@
       <c r="P29" s="12" t="s">
         <v>213</v>
       </c>
-      <c r="Q29" s="12"/>
-    </row>
-    <row r="30" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q29" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R29" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No accuracy/validation data. CHARLS prediction model where self-reported VI is the outcome; the self-report item itself is not evaluated against measured vision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="9">
         <v>29</v>
       </c>
@@ -4591,9 +4849,18 @@
       <c r="P30" s="12" t="s">
         <v>219</v>
       </c>
-      <c r="Q30" s="12"/>
-    </row>
-    <row r="31" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q30" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R30" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No questionnaire/screening item. Develops a battery of performance-based functional tests for low vision; NEI VFQ-25 is only an ancillary measure, not the instrument studied.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="9">
         <v>30</v>
       </c>
@@ -4632,9 +4899,18 @@
       <c r="P31" s="12" t="s">
         <v>224</v>
       </c>
-      <c r="Q31" s="12"/>
-    </row>
-    <row r="32" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q31" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="R31" s="12" t="inlineStr">
+        <is>
+          <t>Adult rehab inpatients: self-reported vision questions (newspaper reading, faces, happiness with vision) tested against VA/CS/VF, sensitivity reported.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="9">
         <v>31</v>
       </c>
@@ -4675,9 +4951,18 @@
       <c r="P32" s="12" t="s">
         <v>230</v>
       </c>
-      <c r="Q32" s="12"/>
-    </row>
-    <row r="33" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q32" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R32" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No accuracy/validation data. Cohort study using self-reported vision questions and contrast sensitivity as risk factors for falls/fractures; questions not evaluated as instruments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="9">
         <v>32</v>
       </c>
@@ -4720,9 +5005,18 @@
       <c r="P33" s="12" t="s">
         <v>236</v>
       </c>
-      <c r="Q33" s="12"/>
-    </row>
-    <row r="34" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q33" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R33" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Wrong population (not adults). Illumination and visual comfort study in schoolchildren with low vision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="9">
         <v>33</v>
       </c>
@@ -4765,9 +5059,18 @@
       <c r="P34" s="12" t="s">
         <v>241</v>
       </c>
-      <c r="Q34" s="12"/>
-    </row>
-    <row r="35" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q34" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R34" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Not about low vision/visual function. Self-reported driving habits in AMD vs controls; the self-report concerns driving behaviour, not a vision questionnaire being evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="9">
         <v>34</v>
       </c>
@@ -4808,9 +5111,18 @@
       <c r="P35" s="12" t="s">
         <v>247</v>
       </c>
-      <c r="Q35" s="12"/>
-    </row>
-    <row r="36" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q35" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R35" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Intervention study only. Economic evaluation of LV rehabilitation vs basic LV services (LOVIT II); VA LV VFQ used only as outcome.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="9">
         <v>35</v>
       </c>
@@ -4853,9 +5165,18 @@
       <c r="P36" s="12" t="s">
         <v>253</v>
       </c>
-      <c r="Q36" s="12"/>
-    </row>
-    <row r="37" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q36" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R36" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No accuracy/validation data. Uveitis study using self-reported visual function as a predictor of anxiety/depression; vision instrument not evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="9">
         <v>36</v>
       </c>
@@ -4896,9 +5217,18 @@
       <c r="P37" s="12" t="s">
         <v>259</v>
       </c>
-      <c r="Q37" s="12"/>
-    </row>
-    <row r="38" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q37" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R37" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Intervention study only. Microperimeter biofeedback fixation training in maculopathy; NEI-VFQ-25 only a pre/post outcome.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="9">
         <v>37</v>
       </c>
@@ -4937,9 +5267,18 @@
       <c r="P38" s="12" t="s">
         <v>265</v>
       </c>
-      <c r="Q38" s="12"/>
-    </row>
-    <row r="39" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q38" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R38" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No accuracy/validation data. Meta-analysis of Dutch VI prevalence using self-report, VA and GP codes; self-report definitions not evaluated for accuracy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="9">
         <v>38</v>
       </c>
@@ -4978,9 +5317,18 @@
       <c r="P39" s="12" t="s">
         <v>271</v>
       </c>
-      <c r="Q39" s="12"/>
-    </row>
-    <row r="40" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q39" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="R39" s="12" t="inlineStr">
+        <is>
+          <t>ESO clinical practice guideline on screening and managing post-stroke visual impairment in adults, including accuracy of vision screening tools; counts as a guideline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="9">
         <v>39</v>
       </c>
@@ -5019,9 +5367,18 @@
       <c r="P40" s="12" t="s">
         <v>277</v>
       </c>
-      <c r="Q40" s="12"/>
-    </row>
-    <row r="41" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q40" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="R40" s="12" t="inlineStr">
+        <is>
+          <t>Rasch psychometric evaluation of the VA-13 self-report blind rehabilitation outcome measure (and clinician FAST) in legally blind veterans.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="9">
         <v>40</v>
       </c>
@@ -5064,9 +5421,18 @@
       <c r="P41" s="12" t="s">
         <v>283</v>
       </c>
-      <c r="Q41" s="12"/>
-    </row>
-    <row r="42" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q41" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="R41" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No questionnaire/screening item. RCT protocol for AI retinal-imaging VI screening; the only questionnaire is patient acceptance of the screening, not a vision self-report.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="9">
         <v>41</v>
       </c>
@@ -5108,8 +5474,13 @@
           <t>Include</t>
         </is>
       </c>
-    </row>
-    <row r="43" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R42" s="12" t="inlineStr">
+        <is>
+          <t>Evidence-based clinical practice guideline for low vision diagnosis/rehabilitation incl. adults; recommends NEI VFQ-25 for follow-up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="9">
         <v>42</v>
       </c>
@@ -5153,8 +5524,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="44" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R43" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No questionnaire/screening item. Braille reading speed correlates in blind adults; no vision self-report tool evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="9">
         <v>43</v>
       </c>
@@ -5198,8 +5574,13 @@
           <t>Maybe</t>
         </is>
       </c>
-    </row>
-    <row r="45" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R44" s="12" t="inlineStr">
+        <is>
+          <t>LVR clinic adults; NEI VFQ-25 related to VA, reading acuity and contrast sensitivity, though main aim is depression screening.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="9">
         <v>44</v>
       </c>
@@ -5243,8 +5624,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="46" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R45" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No questionnaire/screening item. Seasonal affective disorder questionnaire by eye diagnosis; no vision self-report tool evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="9">
         <v>45</v>
       </c>
@@ -5288,8 +5674,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="47" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R46" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No questionnaire/screening item. Facial landmark analysis during a mobile VA test; not a self-report measure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="9">
         <v>46</v>
       </c>
@@ -5331,8 +5722,13 @@
           <t>Include</t>
         </is>
       </c>
-    </row>
-    <row r="48" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R47" s="12" t="inlineStr">
+        <is>
+          <t>Activity Inventory self-reported activity limitation related to VA, VF, contrast and psychosocial factors in VI adults.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="9">
         <v>47</v>
       </c>
@@ -5374,8 +5770,13 @@
           <t>Include</t>
         </is>
       </c>
-    </row>
-    <row r="49" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R48" s="12" t="inlineStr">
+        <is>
+          <t>Dutch ICF Activity Inventory self-reported function related to binocular visual field areas in field-loss patients.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="9">
         <v>48</v>
       </c>
@@ -5417,8 +5818,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="50" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R49" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Intervention study only. Development of a head-mounted low vision aid; no questionnaire validation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="9">
         <v>49</v>
       </c>
@@ -5462,8 +5868,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="51" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R50" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Intervention study only. Pre/post blind rehabilitation outcomes with NEI VFQ; no questionnaire validation or screening data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="9">
         <v>50</v>
       </c>
@@ -5507,8 +5918,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="52" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R51" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No questionnaire/screening item. Clinical/microperimetric predictors of reading speed in AMD; no self-report tool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="9">
         <v>51</v>
       </c>
@@ -5552,8 +5968,13 @@
           <t>Maybe</t>
         </is>
       </c>
-    </row>
-    <row r="53" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R52" s="12" t="inlineStr">
+        <is>
+          <t>Conjoint-analysis tool for LVR priorities in AMD compared with VA, CS and NEI VFQ-25; congress paper, check data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="9">
         <v>52</v>
       </c>
@@ -5597,8 +6018,13 @@
           <t>Maybe</t>
         </is>
       </c>
-    </row>
-    <row r="54" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R53" s="12" t="inlineStr">
+        <is>
+          <t>NEI VFQ-25 related to visual function tests in Parkinson's disease; adult self-report vs vision but non-LVR population.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="9">
         <v>53</v>
       </c>
@@ -5642,8 +6068,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="55" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R54" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Wrong population (not adults). Students with special educational needs (mean age 14); no self-report tool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="9">
         <v>54</v>
       </c>
@@ -5687,8 +6118,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="56" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R55" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Review/opinion/editorial. Meta-analysis of visual impairment and pragmatic impairment; not a questionnaire evaluation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="9">
         <v>55</v>
       </c>
@@ -5730,8 +6166,13 @@
           <t>Include</t>
         </is>
       </c>
-    </row>
-    <row r="57" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R56" s="12" t="inlineStr">
+        <is>
+          <t>Screening questions on falls/mobility and GAL-9 vs VA/CS in maculopathy LVR patients to guide rehabilitation referral.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="9">
         <v>56</v>
       </c>
@@ -5775,8 +6216,13 @@
           <t>Maybe</t>
         </is>
       </c>
-    </row>
-    <row r="58" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R57" s="12" t="inlineStr">
+        <is>
+          <t>LVQOL questionnaire change correlated with VA improvement with low vision aids; possible validity data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="9">
         <v>57</v>
       </c>
@@ -5820,8 +6266,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="59" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R58" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Review/opinion/editorial. Systematic review/meta-analysis of visual impairment and frailty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="9">
         <v>58</v>
       </c>
@@ -5865,8 +6316,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="60" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R59" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No accuracy/validation data. Driving habits survey in low vision patients vs licensure criteria; no questionnaire accuracy or validation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="9">
         <v>59</v>
       </c>
@@ -5910,8 +6366,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="61" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R60" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Wrong population (not adults). Children with Usher syndrome; listening effort focus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="9">
         <v>60</v>
       </c>
@@ -5955,8 +6416,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="62" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R61" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Intervention study only. RCT of a health education programme for AMD; no questionnaire validation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="9">
         <v>61</v>
       </c>
@@ -6000,8 +6466,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="63" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R62" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No accuracy/validation data. Air pollution and self-reported VI epidemiology; self-report item not validated against vision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="9">
         <v>62</v>
       </c>
@@ -6045,8 +6516,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="64" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R63" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Intervention study only. Low vision intervention outcomes in AMD; NEI VFQ-25 used only as outcome.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="9">
         <v>63</v>
       </c>
@@ -6088,8 +6564,13 @@
           <t>Include</t>
         </is>
       </c>
-    </row>
-    <row r="65" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R64" s="12" t="inlineStr">
+        <is>
+          <t>Rasch-analysed 10-item night vision questionnaire compared against measured visual function (LLD, BCVA, microperimetry) in adults with AMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="9">
         <v>64</v>
       </c>
@@ -6133,8 +6614,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="66" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R65" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Intervention study only. Pilot of MP-1 biofeedback rehabilitation in 5 patients; no questionnaire evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="9">
         <v>65</v>
       </c>
@@ -6176,8 +6662,13 @@
           <t>Include</t>
         </is>
       </c>
-    </row>
-    <row r="67" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R66" s="12" t="inlineStr">
+        <is>
+          <t>Rasch evaluation of NEI VFQ-25 item functioning and sensitivity to change in veterans receiving LVR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="9">
         <v>66</v>
       </c>
@@ -6219,8 +6710,13 @@
           <t>Include</t>
         </is>
       </c>
-    </row>
-    <row r="68" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R67" s="12" t="inlineStr">
+        <is>
+          <t>Validation (DIF, responsiveness) of the VA LV VFQ-48 in vision rehabilitation patients.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="9">
         <v>67</v>
       </c>
@@ -6262,8 +6758,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="69" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R68" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Review/opinion/editorial. Narrative review of clinical reading tests; no questionnaire validation reported.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="9">
         <v>68</v>
       </c>
@@ -6307,8 +6808,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="70" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R69" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Intervention study only. MP-1 biofeedback rehabilitation in glaucoma; NEI VFQ-25 used only as an outcome, not validated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="9">
         <v>69</v>
       </c>
@@ -6352,8 +6858,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="71" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R70" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No accuracy/validation data. OCT vs visual function in multiple sclerosis; NEI VFQ collected but not evaluated as an instrument.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="9">
         <v>70</v>
       </c>
@@ -6397,8 +6908,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="72" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R71" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No questionnaire/screening item. Population study linking objectively measured VI to dementia; no self-report vision tool evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="9">
         <v>71</v>
       </c>
@@ -6442,8 +6958,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="73" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R72" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Not about low vision/visual function. Pricing survey of specialists on off-label Avastin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="9">
         <v>72</v>
       </c>
@@ -6485,8 +7006,13 @@
           <t>Include</t>
         </is>
       </c>
-    </row>
-    <row r="74" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R73" s="12" t="inlineStr">
+        <is>
+          <t>Compares responsiveness of IVI and NEI VFQ-25 in low vision patients after vision rehabilitation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="9">
         <v>73</v>
       </c>
@@ -6528,8 +7054,13 @@
           <t>Maybe</t>
         </is>
       </c>
-    </row>
-    <row r="75" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R74" s="12" t="inlineStr">
+        <is>
+          <t>LVR outcome study using Rasch-scaled VA LV VFQ-48 and IVI; unclear whether any measurement-property data are reported.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="9">
         <v>74</v>
       </c>
@@ -6571,8 +7102,13 @@
           <t>Include</t>
         </is>
       </c>
-    </row>
-    <row r="76" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R75" s="12" t="inlineStr">
+        <is>
+          <t>Development and performance of the VA LV VFQ in low vision rehabilitation patients.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="9">
         <v>75</v>
       </c>
@@ -6616,8 +7152,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="77" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R76" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No questionnaire/screening item. Fear-of-falling questionnaire (not a vision instrument) tested as a mediator of physical activity in glaucoma/AMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="9">
         <v>76</v>
       </c>
@@ -6661,8 +7202,13 @@
           <t>Maybe</t>
         </is>
       </c>
-    </row>
-    <row r="78" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R77" s="12" t="inlineStr">
+        <is>
+          <t>Examines construct validity of NEI VFQ-25 against a global QoL item; population and vision comparator unclear from abstract.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="9">
         <v>77</v>
       </c>
@@ -6706,8 +7252,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="79" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R78" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Intervention study only. Biofeedback training in 6 AMD patients; questionnaire used only as an outcome.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="9">
         <v>78</v>
       </c>
@@ -6751,8 +7302,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="80" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R79" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Review/opinion/editorial. Systematic review of Charles Bonnet syndrome prevalence; not about LVR screening questionnaires.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="9">
         <v>79</v>
       </c>
@@ -6794,8 +7350,13 @@
           <t>Include</t>
         </is>
       </c>
-    </row>
-    <row r="81" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R80" s="12" t="inlineStr">
+        <is>
+          <t>Two self-report screening questions (newsprint, face at 12 ft) assessed against examined VI with PPV/NPV in older adults.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="9">
         <v>80</v>
       </c>
@@ -6839,8 +7400,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="82" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R81" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No accuracy/validation data. Population prevalence study of myopic macular degeneration; VF-11 questionnaire used only as an outcome, not evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="9">
         <v>81</v>
       </c>
@@ -6884,8 +7450,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="83" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R82" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Wrong population (not adults). Screening tool for cerebral visual impairment in children aged 3-50 months.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="9">
         <v>82</v>
       </c>
@@ -6929,8 +7500,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="84" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R83" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Review/opinion/editorial. Narrative overview of LVR service principles; no questionnaire data and not a referral guideline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="9">
         <v>83</v>
       </c>
@@ -6974,8 +7550,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="85" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R84" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No questionnaire/screening item. Halo software test of visual discrimination in drivers; driving questionnaire not evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="9">
         <v>84</v>
       </c>
@@ -7017,8 +7598,13 @@
           <t>Maybe</t>
         </is>
       </c>
-    </row>
-    <row r="86" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R85" s="12" t="inlineStr">
+        <is>
+          <t>NEI VFQ-25 correlated with measured visual function in Stargardt disease; small sample, and adult age needs confirming.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="9">
         <v>85</v>
       </c>
@@ -7062,8 +7648,13 @@
           <t>Maybe</t>
         </is>
       </c>
-    </row>
-    <row r="87" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R86" s="12" t="inlineStr">
+        <is>
+          <t>Qualitative content-validity refinement of an LVR outcome instrument (LVIM); no psychometric data, but relevant to LVR tools.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="9">
         <v>86</v>
       </c>
@@ -7105,8 +7696,13 @@
           <t>Include</t>
         </is>
       </c>
-    </row>
-    <row r="88" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R87" s="12" t="inlineStr">
+        <is>
+          <t>Rasch-analysed Participation and Activity Inventory measuring rehabilitative need in adults entering LVR, related to VA and other measures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="9">
         <v>87</v>
       </c>
@@ -7150,8 +7746,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="89" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R88" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No accuracy/validation data. Population study of vision and fear of falling; single self-rated vision item used as exposure, not validated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="9">
         <v>88</v>
       </c>
@@ -7192,11 +7793,16 @@
       </c>
       <c r="Q89" s="12" t="inlineStr">
         <is>
-          <t>Include</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Maybe</t>
+        </is>
+      </c>
+      <c r="R89" s="12" t="inlineStr">
+        <is>
+          <t>Responsiveness and discrimination of the generic EQ-5D tested against the Activity Inventory in LVR patients; measurement-property data, but EQ-5D is not a vision-specific instrument.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="9">
         <v>89</v>
       </c>
@@ -7238,8 +7844,13 @@
           <t>Include</t>
         </is>
       </c>
-    </row>
-    <row r="91" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R90" s="12" t="inlineStr">
+        <is>
+          <t>Rasch-based responsiveness validation of the LVIM-R in adults receiving low vision rehabilitation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="9">
         <v>90</v>
       </c>
@@ -7283,8 +7894,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="92" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R91" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No questionnaire/screening item. Falls and injuries in AMD predicted by clinical vision measures; no self-report tool evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="9">
         <v>91</v>
       </c>
@@ -7328,8 +7944,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="93" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R92" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No questionnaire/screening item. Two-participant study of BCI/eye-tracking typing in ALS; no questionnaire evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="9">
         <v>92</v>
       </c>
@@ -7371,8 +7992,13 @@
           <t>Include</t>
         </is>
       </c>
-    </row>
-    <row r="94" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R93" s="12" t="inlineStr">
+        <is>
+          <t>Screening questions (menu, keyboard) vs measured VA in 385 adults with sensitivity, specificity and AUC; core study.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="9">
         <v>93</v>
       </c>
@@ -7412,8 +8038,13 @@
           <t>Include</t>
         </is>
       </c>
-    </row>
-    <row r="95" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R94" s="12" t="inlineStr">
+        <is>
+          <t>USPSTF systematic review that summarises accuracy of screening questions vs VA testing in older adults.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="9">
         <v>94</v>
       </c>
@@ -7457,8 +8088,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="96" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R95" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Wrong population (not adults). Parent-reported CVI questionnaire in children.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="9">
         <v>95</v>
       </c>
@@ -7502,8 +8138,13 @@
           <t>Include</t>
         </is>
       </c>
-    </row>
-    <row r="97" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R96" s="12" t="inlineStr">
+        <is>
+          <t>Rasch validation of self-reported driving difficulty in 851 low-vision clinic patients, related to VA and CS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="9">
         <v>96</v>
       </c>
@@ -7547,8 +8188,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="98" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R97" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Intervention study only. PRL biofeedback training outcomes; VFQ-25 used only as an outcome measure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="9">
         <v>97</v>
       </c>
@@ -7592,8 +8238,13 @@
           <t>Include</t>
         </is>
       </c>
-    </row>
-    <row r="99" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R98" s="12" t="inlineStr">
+        <is>
+          <t>Develops and Rasch-validates the Spatial Localization Questionnaire against clinical vision tests in visually impaired adults.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="9">
         <v>98</v>
       </c>
@@ -7637,8 +8288,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="100" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R99" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No accuracy/validation data. Driving simulator speed study in cataract; Driver Habits Questionnaire used descriptively without validation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="9">
         <v>99</v>
       </c>
@@ -7682,8 +8338,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="101" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R100" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Intervention study only. RCT and cost-effectiveness of basic LVR; no questionnaire validation or screening data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="9">
         <v>100</v>
       </c>
@@ -7727,8 +8388,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="102" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R101" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No accuracy/validation data. Self-reported VI (NEI-VFQ) as an exposure for cognitive decline; no validation against vision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="9">
         <v>101</v>
       </c>
@@ -7772,8 +8438,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="103" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R102" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Intervention study only. Head-mounted device trial; VA LV VFQ-48 used only as an outcome measure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="9">
         <v>102</v>
       </c>
@@ -7817,8 +8488,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="104" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R103" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Wrong population (not adults). CVI diagnosis and referral guidelines for children aged 18 or under.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="9">
         <v>103</v>
       </c>
@@ -7862,8 +8538,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="105" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R104" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No questionnaire/screening item. Home hazards, measured vision and falls; no self-report vision tool evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="9">
         <v>104</v>
       </c>
@@ -7907,8 +8588,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="106" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R105" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No questionnaire/screening item. Season, sunlight and depressive symptoms in VI; no vision self-report tool evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="9">
         <v>105</v>
       </c>
@@ -7950,8 +8636,13 @@
           <t>Include</t>
         </is>
       </c>
-    </row>
-    <row r="107" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R106" s="12" t="inlineStr">
+        <is>
+          <t>Validation of the Italian VA LV VFQ-48 in LVR patients, with reliability and correlation with VA and reading.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="9">
         <v>106</v>
       </c>
@@ -7995,8 +8686,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="108" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R107" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No accuracy/validation data. Gaze perception task study; brief questionnaire used as a predictor, not validated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="9">
         <v>107</v>
       </c>
@@ -8040,8 +8736,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="109" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R108" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No accuracy/validation data. Determinants-of-QoL regression in LV clinic patients; questionnaires used as outcomes, not validated or tested for accuracy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="9">
         <v>108</v>
       </c>
@@ -8083,8 +8784,13 @@
           <t>Maybe</t>
         </is>
       </c>
-    </row>
-    <row r="110" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R109" s="12" t="inlineStr">
+        <is>
+          <t>Population study relating NEI VFQ-25 scores to measured acuity and eye disease incl. glaucoma; may give known-groups validity data for a full-length questionnaire.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="9">
         <v>109</v>
       </c>
@@ -8128,8 +8834,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="111" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R110" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No questionnaire/screening item. Work ability and psychosocial work questionnaires in low vision; no vision self-report tool evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="9">
         <v>110</v>
       </c>
@@ -8171,8 +8882,13 @@
           <t>Include</t>
         </is>
       </c>
-    </row>
-    <row r="112" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R111" s="12" t="inlineStr">
+        <is>
+          <t>Glaucoma patients' visual disability questionnaire correlated against Humphrey VF and VA (glaucoma PROM vs measured vision).</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="9">
         <v>111</v>
       </c>
@@ -8216,8 +8932,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="113" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R112" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No questionnaire/screening item. Falls vs visual function in low vision; ADL questionnaire only a covariate, not evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="9">
         <v>112</v>
       </c>
@@ -8259,8 +8980,13 @@
           <t>Include</t>
         </is>
       </c>
-    </row>
-    <row r="114" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R113" s="12" t="inlineStr">
+        <is>
+          <t>Adults &gt;50 in primary care; compares time to administer the Functional Vision Screening Questionnaire with chart tests (feasibility outcome in PICO).</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="9">
         <v>113</v>
       </c>
@@ -8304,8 +9030,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="115" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R114" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Wrong population (not adults). Parent-reported CVI screening questionnaires in children.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="9">
         <v>114</v>
       </c>
@@ -8349,8 +9080,13 @@
           <t>Include</t>
         </is>
       </c>
-    </row>
-    <row r="116" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R115" s="12" t="inlineStr">
+        <is>
+          <t>Psychometric validation (reliability, known-groups by VA) of Thai vision bolt-on EQ-5D in visually impaired participants.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="9">
         <v>115</v>
       </c>
@@ -8394,8 +9130,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="117" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R116" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No accuracy/validation data. Translation and cultural adaptation of LVQOL only; psychometric validation deferred to a later study.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="9">
         <v>116</v>
       </c>
@@ -8439,8 +9180,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="118" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R117" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No questionnaire/screening item. Cohort study of measured VA and mortality; no self-report tool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="9">
         <v>117</v>
       </c>
@@ -8482,8 +9228,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="119" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R118" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Not about low vision/visual function. Symptom questionnaire to differentiate dry eye from other diagnoses; not judged against vision impairment or LVR need.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="9">
         <v>118</v>
       </c>
@@ -8527,8 +9278,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="120" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R119" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Wrong population (not adults). Validation of an iPad CVI screening app in children aged 5-18.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="9">
         <v>119</v>
       </c>
@@ -8570,8 +9326,13 @@
           <t>Include</t>
         </is>
       </c>
-    </row>
-    <row r="121" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R120" s="12" t="inlineStr">
+        <is>
+          <t>Validation of Spanish LVQOL with reliability, IRT and sensitivity/specificity cut-off for detecting visual impairment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="9">
         <v>120</v>
       </c>
@@ -8613,8 +9374,13 @@
           <t>Include</t>
         </is>
       </c>
-    </row>
-    <row r="122" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R121" s="12" t="inlineStr">
+        <is>
+          <t>Self-reported mobility questionnaire validated against VA, CS and VF in low vision patients, proposed as guide for O&amp;M referral.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="9">
         <v>121</v>
       </c>
@@ -8656,8 +9422,13 @@
           <t>Maybe</t>
         </is>
       </c>
-    </row>
-    <row r="123" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R122" s="12" t="inlineStr">
+        <is>
+          <t>Visual difficulty questionnaire with factor and discriminant analysis between low-vision and nonimpaired older drivers; unclear if accuracy data reported.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="9">
         <v>122</v>
       </c>
@@ -8699,8 +9470,13 @@
           <t>Include</t>
         </is>
       </c>
-    </row>
-    <row r="124" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R123" s="12" t="inlineStr">
+        <is>
+          <t>LVQOL in advanced glaucoma with low vision related to VA, MD and edge detection with AUROC analysis (glaucoma PROM study).</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="9">
         <v>123</v>
       </c>
@@ -8744,8 +9520,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="125" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R124" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No questionnaire/screening item. Postural sway vs visual field loss in glaucoma; no self-report vision tool evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="9">
         <v>124</v>
       </c>
@@ -8789,8 +9570,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="126" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R125" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No accuracy/validation data. Self-reported VFQ used only as a predictor of physical performance decline; not validated against vision measures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="9">
         <v>125</v>
       </c>
@@ -8834,8 +9620,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="127" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R126" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No accuracy/validation data. Self-reported visual difficulty used as an exposure for sleep outcomes; no accuracy or validation of the item.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="9">
         <v>126</v>
       </c>
@@ -8879,8 +9670,13 @@
           <t>Exclude</t>
         </is>
       </c>
-    </row>
-    <row r="128" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R127" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: Not about low vision/visual function. Self-assessed driving skill vs on-road evaluation in bioptic drivers; not a vision/LVR-need screening tool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="9">
         <v>127</v>
       </c>
@@ -8924,9 +9720,14 @@
           <t>Exclude</t>
         </is>
       </c>
+      <c r="R128" s="12" t="inlineStr">
+        <is>
+          <t>Exclusion reason: No questionnaire/screening item. Survey of orthoptists' LVR practice for AMD in France; no patient self-report tool or referral guideline.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q128" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:R128" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <conditionalFormatting sqref="H2:H128">
     <cfRule type="expression" dxfId="8" priority="2">
       <formula>H2="Include"</formula>

</xml_diff>

<commit_message>
Grab 4 more missing articles; split out independent AI exclusion reason
Move the exclusion reason out of the independent AI rationale text into
its own "Independent exclusion reason (AI)" column, and regenerate the
Screening CSV.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/LVR_screening_sheet_2.xlsx
+++ b/data/LVR_screening_sheet_2.xlsx
@@ -3243,7 +3243,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:R128"/>
+  <dimension ref="A1:S128"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -3263,10 +3263,11 @@
     <col min="15" max="15" width="28" customWidth="1"/>
     <col min="16" max="16" width="55" customWidth="1"/>
     <col min="17" max="17" width="16" customWidth="1"/>
-    <col min="18" max="18" width="60" customWidth="1"/>
+    <col min="18" max="18" width="28" customWidth="1"/>
+    <col min="19" max="19" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:19" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
         <v>29</v>
       </c>
@@ -3322,11 +3323,16 @@
       </c>
       <c r="R1" s="8" t="inlineStr">
         <is>
+          <t>Independent exclusion reason (AI)</t>
+        </is>
+      </c>
+      <c r="S1" s="8" t="inlineStr">
+        <is>
           <t>Independent rationale (AI)</t>
         </is>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="9">
         <v>1</v>
       </c>
@@ -3372,11 +3378,16 @@
       </c>
       <c r="R2" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Wrong population (not adults). Study of social support for high school students with visual impairment; children only and no self-report vision instrument evaluated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Wrong population (not adults)</t>
+        </is>
+      </c>
+      <c r="S2" s="12" t="inlineStr">
+        <is>
+          <t>Study of social support for high school students with visual impairment; children only and no self-report vision instrument evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="9">
         <v>2</v>
       </c>
@@ -3426,11 +3437,16 @@
       </c>
       <c r="R3" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Other (see notes). Case series of 2 patients fitted with multifocal RGP lenses; VFQ-25 used only as an outcome. Case series are excluded.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Other (see notes)</t>
+        </is>
+      </c>
+      <c r="S3" s="12" t="inlineStr">
+        <is>
+          <t>Case series of 2 patients fitted with multifocal RGP lenses; VFQ-25 used only as an outcome. Case series are excluded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="9">
         <v>3</v>
       </c>
@@ -3480,11 +3496,16 @@
       </c>
       <c r="R4" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No accuracy/validation data. Cross-sectional study of factors linked to adjustment to vision loss; AS-WAS and self-reported activity limitation are used as outcome/predictors, not evaluated as instruments.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No accuracy/validation data</t>
+        </is>
+      </c>
+      <c r="S4" s="12" t="inlineStr">
+        <is>
+          <t>Cross-sectional study of factors linked to adjustment to vision loss; AS-WAS and self-reported activity limitation are used as outcome/predictors, not evaluated as instruments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="9">
         <v>4</v>
       </c>
@@ -3534,11 +3555,16 @@
       </c>
       <c r="R5" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Review/opinion/editorial. Narrative overview of preferred retinal locus and biofeedback training; no questionnaire evaluation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Review/opinion/editorial</t>
+        </is>
+      </c>
+      <c r="S5" s="12" t="inlineStr">
+        <is>
+          <t>Narrative overview of preferred retinal locus and biofeedback training; no questionnaire evaluation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="9">
         <v>5</v>
       </c>
@@ -3582,13 +3608,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R6" s="12" t="inlineStr">
+      <c r="R6" s="12"/>
+      <c r="S6" s="12" t="inlineStr">
         <is>
           <t>Rasch analysis of the APEDS-VFQ visual function questionnaire in 351 visually impaired adults; psychometric validation of a self-report vision instrument.</t>
         </is>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="9">
         <v>6</v>
       </c>
@@ -3638,11 +3665,16 @@
       </c>
       <c r="R7" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No accuracy/validation data. Nursing-home teleophthalmology study; the NHVQoL questionnaire is administered descriptively, with no accuracy or psychometric evaluation of it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No accuracy/validation data</t>
+        </is>
+      </c>
+      <c r="S7" s="12" t="inlineStr">
+        <is>
+          <t>Nursing-home teleophthalmology study; the NHVQoL questionnaire is administered descriptively, with no accuracy or psychometric evaluation of it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9">
         <v>7</v>
       </c>
@@ -3692,11 +3724,16 @@
       </c>
       <c r="R8" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No questionnaire/screening item. Survey of teachers on assistive technology for blind and low-vision students; no self-report vision instrument is evaluated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="S8" s="12" t="inlineStr">
+        <is>
+          <t>Survey of teachers on assistive technology for blind and low-vision students; no self-report vision instrument is evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="9">
         <v>8</v>
       </c>
@@ -3746,11 +3783,16 @@
       </c>
       <c r="R9" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No questionnaire/screening item. UK Biobank cohort linking measured visual acuity to incident Parkinson's disease; no self-report vision instrument.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="S9" s="12" t="inlineStr">
+        <is>
+          <t>UK Biobank cohort linking measured visual acuity to incident Parkinson's disease; no self-report vision instrument.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="9">
         <v>9</v>
       </c>
@@ -3800,11 +3842,16 @@
       </c>
       <c r="R10" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No questionnaire/screening item. NHATS analysis of measured VI (acuity, contrast) and homebound status; no self-report vision instrument is evaluated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="S10" s="12" t="inlineStr">
+        <is>
+          <t>NHATS analysis of measured VI (acuity, contrast) and homebound status; no self-report vision instrument is evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="9">
         <v>10</v>
       </c>
@@ -3854,11 +3901,16 @@
       </c>
       <c r="R11" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No accuracy/validation data. Epidemiological study of diet, mold exposure and VI in older Chinese adults; the VI assessment is only an outcome and is not itself evaluated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No accuracy/validation data</t>
+        </is>
+      </c>
+      <c r="S11" s="12" t="inlineStr">
+        <is>
+          <t>Epidemiological study of diet, mold exposure and VI in older Chinese adults; the VI assessment is only an outcome and is not itself evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="9">
         <v>11</v>
       </c>
@@ -3908,11 +3960,16 @@
       </c>
       <c r="R12" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Not about low vision/visual function. Usability questionnaire for an e-learning course and colour-contrast check; the self-report is about learning preferences, not vision.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Not about low vision/visual function</t>
+        </is>
+      </c>
+      <c r="S12" s="12" t="inlineStr">
+        <is>
+          <t>Usability questionnaire for an e-learning course and colour-contrast check; the self-report is about learning preferences, not vision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="9">
         <v>12</v>
       </c>
@@ -3958,13 +4015,14 @@
           <t>Maybe</t>
         </is>
       </c>
-      <c r="R13" s="12" t="inlineStr">
+      <c r="R13" s="12"/>
+      <c r="S13" s="12" t="inlineStr">
         <is>
           <t>LVROS baseline of 764 LVR patients; reports that VA correlates poorly with self-reported vision quality, relevant to LVR referral. Unclear if any instrument is formally evaluated.</t>
         </is>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="9">
         <v>13</v>
       </c>
@@ -4014,11 +4072,16 @@
       </c>
       <c r="R14" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Intervention study only. Evaluation of a head-mounted electronic low vision aid; the questionnaire only records willingness to use the device.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Intervention study only</t>
+        </is>
+      </c>
+      <c r="S14" s="12" t="inlineStr">
+        <is>
+          <t>Evaluation of a head-mounted electronic low vision aid; the questionnaire only records willingness to use the device.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="9">
         <v>14</v>
       </c>
@@ -4066,11 +4129,16 @@
       </c>
       <c r="R15" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Intervention study only. Pilot study of VEP biofeedback rehabilitation in AMD; VFQ-25 used only as an outcome measure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Intervention study only</t>
+        </is>
+      </c>
+      <c r="S15" s="12" t="inlineStr">
+        <is>
+          <t>Pilot study of VEP biofeedback rehabilitation in AMD; VFQ-25 used only as an outcome measure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="9">
         <v>15</v>
       </c>
@@ -4120,11 +4188,16 @@
       </c>
       <c r="R16" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Wrong population (not adults). Review of paediatric assessment of cerebral visual impairment; children only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Wrong population (not adults)</t>
+        </is>
+      </c>
+      <c r="S16" s="12" t="inlineStr">
+        <is>
+          <t>Review of paediatric assessment of cerebral visual impairment; children only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="9">
         <v>16</v>
       </c>
@@ -4172,11 +4245,16 @@
       </c>
       <c r="R17" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No accuracy/validation data. Chart review of glaucoma patients attending vision rehab; self-reported ADL difficulty only described alongside BCVA/VF/CS, intake instrument not evaluated. Useful background on glaucoma LVR referral.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No accuracy/validation data</t>
+        </is>
+      </c>
+      <c r="S17" s="12" t="inlineStr">
+        <is>
+          <t>Chart review of glaucoma patients attending vision rehab; self-reported ADL difficulty only described alongside BCVA/VF/CS, intake instrument not evaluated. Useful background on glaucoma LVR referral.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="9">
         <v>17</v>
       </c>
@@ -4226,11 +4304,16 @@
       </c>
       <c r="R18" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Intervention study only. Outcomes of mobile-clinic LVR measured with the Activity Inventory; MCID used to judge treatment effect, not to evaluate the instrument.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Intervention study only</t>
+        </is>
+      </c>
+      <c r="S18" s="12" t="inlineStr">
+        <is>
+          <t>Outcomes of mobile-clinic LVR measured with the Activity Inventory; MCID used to judge treatment effect, not to evaluate the instrument.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="9">
         <v>18</v>
       </c>
@@ -4278,11 +4361,16 @@
       </c>
       <c r="R19" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Intervention study only. LVROS outcomes of usual LVR care measured with the Activity Inventory; MCID used to quantify rehab effect, not measurement properties.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Intervention study only</t>
+        </is>
+      </c>
+      <c r="S19" s="12" t="inlineStr">
+        <is>
+          <t>LVROS outcomes of usual LVR care measured with the Activity Inventory; MCID used to quantify rehab effect, not measurement properties.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="9">
         <v>19</v>
       </c>
@@ -4332,11 +4420,16 @@
       </c>
       <c r="R20" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No accuracy/validation data. Path analysis of cognitive appraisals, distress and self-reported disability in LVR patients; questionnaires used as predictors/outcomes, not evaluated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No accuracy/validation data</t>
+        </is>
+      </c>
+      <c r="S20" s="12" t="inlineStr">
+        <is>
+          <t>Path analysis of cognitive appraisals, distress and self-reported disability in LVR patients; questionnaires used as predictors/outcomes, not evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="9">
         <v>20</v>
       </c>
@@ -4384,11 +4477,16 @@
       </c>
       <c r="R21" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Review/opinion/editorial. Narrative review of low vision examination and rehabilitation stages; no original questionnaire data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Review/opinion/editorial</t>
+        </is>
+      </c>
+      <c r="S21" s="12" t="inlineStr">
+        <is>
+          <t>Narrative review of low vision examination and rehabilitation stages; no original questionnaire data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="9">
         <v>21</v>
       </c>
@@ -4434,13 +4532,14 @@
           <t>Maybe</t>
         </is>
       </c>
-      <c r="R22" s="12" t="inlineStr">
+      <c r="R22" s="12"/>
+      <c r="S22" s="12" t="inlineStr">
         <is>
           <t>Cochrane review of RCTs in which self-reported vision questions were the community screening tool; reports the effect of such screening on vision (not accuracy), relevant to clinical use.</t>
         </is>
       </c>
     </row>
-    <row r="23" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="9">
         <v>22</v>
       </c>
@@ -4490,11 +4589,16 @@
       </c>
       <c r="R23" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No questionnaire/screening item. Compares short visual acuity charts against clinic VA in older adults; performance tests only, no self-report instrument.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="S23" s="12" t="inlineStr">
+        <is>
+          <t>Compares short visual acuity charts against clinic VA in older adults; performance tests only, no self-report instrument.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="9">
         <v>23</v>
       </c>
@@ -4540,13 +4644,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R24" s="12" t="inlineStr">
+      <c r="R24" s="12"/>
+      <c r="S24" s="12" t="inlineStr">
         <is>
           <t>NHATS older adults: self-reported visual difficulty evaluated against measured VA and contrast sensitivity with AUC, sensitivity and specificity.</t>
         </is>
       </c>
     </row>
-    <row r="25" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="9">
         <v>24</v>
       </c>
@@ -4596,11 +4701,16 @@
       </c>
       <c r="R25" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Intervention study only. RCT protocol on cost-effectiveness of basic vision rehabilitation; Activity Inventory used only as primary outcome.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Intervention study only</t>
+        </is>
+      </c>
+      <c r="S25" s="12" t="inlineStr">
+        <is>
+          <t>RCT protocol on cost-effectiveness of basic vision rehabilitation; Activity Inventory used only as primary outcome.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="9">
         <v>25</v>
       </c>
@@ -4650,11 +4760,16 @@
       </c>
       <c r="R26" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Not about low vision/visual function. PHQ-2 depression screening acceptability in LVR/eye-care clients; the screened construct is depression, not vision or LVR need.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Not about low vision/visual function</t>
+        </is>
+      </c>
+      <c r="S26" s="12" t="inlineStr">
+        <is>
+          <t>PHQ-2 depression screening acceptability in LVR/eye-care clients; the screened construct is depression, not vision or LVR need.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="9">
         <v>26</v>
       </c>
@@ -4698,13 +4813,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R27" s="12" t="inlineStr">
+      <c r="R27" s="12"/>
+      <c r="S27" s="12" t="inlineStr">
         <is>
           <t>Development and psychometric validation (internal consistency, reliability, known-groups, responsiveness) of the LVQOL in low vision patients.</t>
         </is>
       </c>
     </row>
-    <row r="28" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="9">
         <v>27</v>
       </c>
@@ -4748,13 +4864,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R28" s="12" t="inlineStr">
+      <c r="R28" s="12"/>
+      <c r="S28" s="12" t="inlineStr">
         <is>
           <t>Validates Visual Impairment as a Risk for Falls Questionnaire items (e.g. reading, faces) against oculo-visual exam, with sensitivity and specificity.</t>
         </is>
       </c>
     </row>
-    <row r="29" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="9">
         <v>28</v>
       </c>
@@ -4804,11 +4921,16 @@
       </c>
       <c r="R29" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No accuracy/validation data. CHARLS prediction model where self-reported VI is the outcome; the self-report item itself is not evaluated against measured vision.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No accuracy/validation data</t>
+        </is>
+      </c>
+      <c r="S29" s="12" t="inlineStr">
+        <is>
+          <t>CHARLS prediction model where self-reported VI is the outcome; the self-report item itself is not evaluated against measured vision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="9">
         <v>29</v>
       </c>
@@ -4856,11 +4978,16 @@
       </c>
       <c r="R30" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No questionnaire/screening item. Develops a battery of performance-based functional tests for low vision; NEI VFQ-25 is only an ancillary measure, not the instrument studied.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="S30" s="12" t="inlineStr">
+        <is>
+          <t>Develops a battery of performance-based functional tests for low vision; NEI VFQ-25 is only an ancillary measure, not the instrument studied.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="9">
         <v>30</v>
       </c>
@@ -4904,13 +5031,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R31" s="12" t="inlineStr">
+      <c r="R31" s="12"/>
+      <c r="S31" s="12" t="inlineStr">
         <is>
           <t>Adult rehab inpatients: self-reported vision questions (newspaper reading, faces, happiness with vision) tested against VA/CS/VF, sensitivity reported.</t>
         </is>
       </c>
     </row>
-    <row r="32" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="9">
         <v>31</v>
       </c>
@@ -4958,11 +5086,16 @@
       </c>
       <c r="R32" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No accuracy/validation data. Cohort study using self-reported vision questions and contrast sensitivity as risk factors for falls/fractures; questions not evaluated as instruments.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No accuracy/validation data</t>
+        </is>
+      </c>
+      <c r="S32" s="12" t="inlineStr">
+        <is>
+          <t>Cohort study using self-reported vision questions and contrast sensitivity as risk factors for falls/fractures; questions not evaluated as instruments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="9">
         <v>32</v>
       </c>
@@ -5012,11 +5145,16 @@
       </c>
       <c r="R33" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Wrong population (not adults). Illumination and visual comfort study in schoolchildren with low vision.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Wrong population (not adults)</t>
+        </is>
+      </c>
+      <c r="S33" s="12" t="inlineStr">
+        <is>
+          <t>Illumination and visual comfort study in schoolchildren with low vision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="9">
         <v>33</v>
       </c>
@@ -5066,11 +5204,16 @@
       </c>
       <c r="R34" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Not about low vision/visual function. Self-reported driving habits in AMD vs controls; the self-report concerns driving behaviour, not a vision questionnaire being evaluated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Not about low vision/visual function</t>
+        </is>
+      </c>
+      <c r="S34" s="12" t="inlineStr">
+        <is>
+          <t>Self-reported driving habits in AMD vs controls; the self-report concerns driving behaviour, not a vision questionnaire being evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="9">
         <v>34</v>
       </c>
@@ -5118,11 +5261,16 @@
       </c>
       <c r="R35" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Intervention study only. Economic evaluation of LV rehabilitation vs basic LV services (LOVIT II); VA LV VFQ used only as outcome.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Intervention study only</t>
+        </is>
+      </c>
+      <c r="S35" s="12" t="inlineStr">
+        <is>
+          <t>Economic evaluation of LV rehabilitation vs basic LV services (LOVIT II); VA LV VFQ used only as outcome.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="9">
         <v>35</v>
       </c>
@@ -5172,11 +5320,16 @@
       </c>
       <c r="R36" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No accuracy/validation data. Uveitis study using self-reported visual function as a predictor of anxiety/depression; vision instrument not evaluated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No accuracy/validation data</t>
+        </is>
+      </c>
+      <c r="S36" s="12" t="inlineStr">
+        <is>
+          <t>Uveitis study using self-reported visual function as a predictor of anxiety/depression; vision instrument not evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="9">
         <v>36</v>
       </c>
@@ -5224,11 +5377,16 @@
       </c>
       <c r="R37" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Intervention study only. Microperimeter biofeedback fixation training in maculopathy; NEI-VFQ-25 only a pre/post outcome.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Intervention study only</t>
+        </is>
+      </c>
+      <c r="S37" s="12" t="inlineStr">
+        <is>
+          <t>Microperimeter biofeedback fixation training in maculopathy; NEI-VFQ-25 only a pre/post outcome.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="9">
         <v>37</v>
       </c>
@@ -5274,11 +5432,16 @@
       </c>
       <c r="R38" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No accuracy/validation data. Meta-analysis of Dutch VI prevalence using self-report, VA and GP codes; self-report definitions not evaluated for accuracy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No accuracy/validation data</t>
+        </is>
+      </c>
+      <c r="S38" s="12" t="inlineStr">
+        <is>
+          <t>Meta-analysis of Dutch VI prevalence using self-report, VA and GP codes; self-report definitions not evaluated for accuracy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="9">
         <v>38</v>
       </c>
@@ -5322,13 +5485,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R39" s="12" t="inlineStr">
+      <c r="R39" s="12"/>
+      <c r="S39" s="12" t="inlineStr">
         <is>
           <t>ESO clinical practice guideline on screening and managing post-stroke visual impairment in adults, including accuracy of vision screening tools; counts as a guideline.</t>
         </is>
       </c>
     </row>
-    <row r="40" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="9">
         <v>39</v>
       </c>
@@ -5372,13 +5536,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R40" s="12" t="inlineStr">
+      <c r="R40" s="12"/>
+      <c r="S40" s="12" t="inlineStr">
         <is>
           <t>Rasch psychometric evaluation of the VA-13 self-report blind rehabilitation outcome measure (and clinician FAST) in legally blind veterans.</t>
         </is>
       </c>
     </row>
-    <row r="41" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="9">
         <v>40</v>
       </c>
@@ -5428,11 +5593,16 @@
       </c>
       <c r="R41" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No questionnaire/screening item. RCT protocol for AI retinal-imaging VI screening; the only questionnaire is patient acceptance of the screening, not a vision self-report.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="S41" s="12" t="inlineStr">
+        <is>
+          <t>RCT protocol for AI retinal-imaging VI screening; the only questionnaire is patient acceptance of the screening, not a vision self-report.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="9">
         <v>41</v>
       </c>
@@ -5474,13 +5644,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R42" s="12" t="inlineStr">
+      <c r="R42" s="12"/>
+      <c r="S42" s="12" t="inlineStr">
         <is>
           <t>Evidence-based clinical practice guideline for low vision diagnosis/rehabilitation incl. adults; recommends NEI VFQ-25 for follow-up.</t>
         </is>
       </c>
     </row>
-    <row r="43" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="9">
         <v>42</v>
       </c>
@@ -5526,11 +5697,16 @@
       </c>
       <c r="R43" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No questionnaire/screening item. Braille reading speed correlates in blind adults; no vision self-report tool evaluated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="S43" s="12" t="inlineStr">
+        <is>
+          <t>Braille reading speed correlates in blind adults; no vision self-report tool evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="9">
         <v>43</v>
       </c>
@@ -5574,13 +5750,14 @@
           <t>Maybe</t>
         </is>
       </c>
-      <c r="R44" s="12" t="inlineStr">
+      <c r="R44" s="12"/>
+      <c r="S44" s="12" t="inlineStr">
         <is>
           <t>LVR clinic adults; NEI VFQ-25 related to VA, reading acuity and contrast sensitivity, though main aim is depression screening.</t>
         </is>
       </c>
     </row>
-    <row r="45" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="9">
         <v>44</v>
       </c>
@@ -5626,11 +5803,16 @@
       </c>
       <c r="R45" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No questionnaire/screening item. Seasonal affective disorder questionnaire by eye diagnosis; no vision self-report tool evaluated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="S45" s="12" t="inlineStr">
+        <is>
+          <t>Seasonal affective disorder questionnaire by eye diagnosis; no vision self-report tool evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="9">
         <v>45</v>
       </c>
@@ -5676,11 +5858,16 @@
       </c>
       <c r="R46" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No questionnaire/screening item. Facial landmark analysis during a mobile VA test; not a self-report measure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="S46" s="12" t="inlineStr">
+        <is>
+          <t>Facial landmark analysis during a mobile VA test; not a self-report measure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="9">
         <v>46</v>
       </c>
@@ -5722,13 +5909,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R47" s="12" t="inlineStr">
+      <c r="R47" s="12"/>
+      <c r="S47" s="12" t="inlineStr">
         <is>
           <t>Activity Inventory self-reported activity limitation related to VA, VF, contrast and psychosocial factors in VI adults.</t>
         </is>
       </c>
     </row>
-    <row r="48" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="9">
         <v>47</v>
       </c>
@@ -5770,13 +5958,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R48" s="12" t="inlineStr">
+      <c r="R48" s="12"/>
+      <c r="S48" s="12" t="inlineStr">
         <is>
           <t>Dutch ICF Activity Inventory self-reported function related to binocular visual field areas in field-loss patients.</t>
         </is>
       </c>
     </row>
-    <row r="49" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="9">
         <v>48</v>
       </c>
@@ -5820,11 +6009,16 @@
       </c>
       <c r="R49" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Intervention study only. Development of a head-mounted low vision aid; no questionnaire validation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Intervention study only</t>
+        </is>
+      </c>
+      <c r="S49" s="12" t="inlineStr">
+        <is>
+          <t>Development of a head-mounted low vision aid; no questionnaire validation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="9">
         <v>49</v>
       </c>
@@ -5870,11 +6064,16 @@
       </c>
       <c r="R50" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Intervention study only. Pre/post blind rehabilitation outcomes with NEI VFQ; no questionnaire validation or screening data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Intervention study only</t>
+        </is>
+      </c>
+      <c r="S50" s="12" t="inlineStr">
+        <is>
+          <t>Pre/post blind rehabilitation outcomes with NEI VFQ; no questionnaire validation or screening data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="9">
         <v>50</v>
       </c>
@@ -5920,11 +6119,16 @@
       </c>
       <c r="R51" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No questionnaire/screening item. Clinical/microperimetric predictors of reading speed in AMD; no self-report tool.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="S51" s="12" t="inlineStr">
+        <is>
+          <t>Clinical/microperimetric predictors of reading speed in AMD; no self-report tool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="9">
         <v>51</v>
       </c>
@@ -5968,13 +6172,14 @@
           <t>Maybe</t>
         </is>
       </c>
-      <c r="R52" s="12" t="inlineStr">
+      <c r="R52" s="12"/>
+      <c r="S52" s="12" t="inlineStr">
         <is>
           <t>Conjoint-analysis tool for LVR priorities in AMD compared with VA, CS and NEI VFQ-25; congress paper, check data.</t>
         </is>
       </c>
     </row>
-    <row r="53" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="9">
         <v>52</v>
       </c>
@@ -6018,13 +6223,14 @@
           <t>Maybe</t>
         </is>
       </c>
-      <c r="R53" s="12" t="inlineStr">
+      <c r="R53" s="12"/>
+      <c r="S53" s="12" t="inlineStr">
         <is>
           <t>NEI VFQ-25 related to visual function tests in Parkinson's disease; adult self-report vs vision but non-LVR population.</t>
         </is>
       </c>
     </row>
-    <row r="54" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="9">
         <v>53</v>
       </c>
@@ -6070,11 +6276,16 @@
       </c>
       <c r="R54" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Wrong population (not adults). Students with special educational needs (mean age 14); no self-report tool.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Wrong population (not adults)</t>
+        </is>
+      </c>
+      <c r="S54" s="12" t="inlineStr">
+        <is>
+          <t>Students with special educational needs (mean age 14); no self-report tool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="9">
         <v>54</v>
       </c>
@@ -6120,11 +6331,16 @@
       </c>
       <c r="R55" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Review/opinion/editorial. Meta-analysis of visual impairment and pragmatic impairment; not a questionnaire evaluation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Review/opinion/editorial</t>
+        </is>
+      </c>
+      <c r="S55" s="12" t="inlineStr">
+        <is>
+          <t>Meta-analysis of visual impairment and pragmatic impairment; not a questionnaire evaluation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="9">
         <v>55</v>
       </c>
@@ -6166,13 +6382,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R56" s="12" t="inlineStr">
+      <c r="R56" s="12"/>
+      <c r="S56" s="12" t="inlineStr">
         <is>
           <t>Screening questions on falls/mobility and GAL-9 vs VA/CS in maculopathy LVR patients to guide rehabilitation referral.</t>
         </is>
       </c>
     </row>
-    <row r="57" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="9">
         <v>56</v>
       </c>
@@ -6216,13 +6433,14 @@
           <t>Maybe</t>
         </is>
       </c>
-      <c r="R57" s="12" t="inlineStr">
+      <c r="R57" s="12"/>
+      <c r="S57" s="12" t="inlineStr">
         <is>
           <t>LVQOL questionnaire change correlated with VA improvement with low vision aids; possible validity data.</t>
         </is>
       </c>
     </row>
-    <row r="58" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="9">
         <v>57</v>
       </c>
@@ -6268,11 +6486,16 @@
       </c>
       <c r="R58" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Review/opinion/editorial. Systematic review/meta-analysis of visual impairment and frailty.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Review/opinion/editorial</t>
+        </is>
+      </c>
+      <c r="S58" s="12" t="inlineStr">
+        <is>
+          <t>Systematic review/meta-analysis of visual impairment and frailty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="9">
         <v>58</v>
       </c>
@@ -6318,11 +6541,16 @@
       </c>
       <c r="R59" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No accuracy/validation data. Driving habits survey in low vision patients vs licensure criteria; no questionnaire accuracy or validation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No accuracy/validation data</t>
+        </is>
+      </c>
+      <c r="S59" s="12" t="inlineStr">
+        <is>
+          <t>Driving habits survey in low vision patients vs licensure criteria; no questionnaire accuracy or validation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="9">
         <v>59</v>
       </c>
@@ -6368,11 +6596,16 @@
       </c>
       <c r="R60" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Wrong population (not adults). Children with Usher syndrome; listening effort focus.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Wrong population (not adults)</t>
+        </is>
+      </c>
+      <c r="S60" s="12" t="inlineStr">
+        <is>
+          <t>Children with Usher syndrome; listening effort focus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="9">
         <v>60</v>
       </c>
@@ -6418,11 +6651,16 @@
       </c>
       <c r="R61" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Intervention study only. RCT of a health education programme for AMD; no questionnaire validation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Intervention study only</t>
+        </is>
+      </c>
+      <c r="S61" s="12" t="inlineStr">
+        <is>
+          <t>RCT of a health education programme for AMD; no questionnaire validation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="9">
         <v>61</v>
       </c>
@@ -6468,11 +6706,16 @@
       </c>
       <c r="R62" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No accuracy/validation data. Air pollution and self-reported VI epidemiology; self-report item not validated against vision.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No accuracy/validation data</t>
+        </is>
+      </c>
+      <c r="S62" s="12" t="inlineStr">
+        <is>
+          <t>Air pollution and self-reported VI epidemiology; self-report item not validated against vision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="9">
         <v>62</v>
       </c>
@@ -6518,11 +6761,16 @@
       </c>
       <c r="R63" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Intervention study only. Low vision intervention outcomes in AMD; NEI VFQ-25 used only as outcome.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Intervention study only</t>
+        </is>
+      </c>
+      <c r="S63" s="12" t="inlineStr">
+        <is>
+          <t>Low vision intervention outcomes in AMD; NEI VFQ-25 used only as outcome.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="9">
         <v>63</v>
       </c>
@@ -6564,13 +6812,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R64" s="12" t="inlineStr">
+      <c r="R64" s="12"/>
+      <c r="S64" s="12" t="inlineStr">
         <is>
           <t>Rasch-analysed 10-item night vision questionnaire compared against measured visual function (LLD, BCVA, microperimetry) in adults with AMD.</t>
         </is>
       </c>
     </row>
-    <row r="65" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="9">
         <v>64</v>
       </c>
@@ -6616,11 +6865,16 @@
       </c>
       <c r="R65" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Intervention study only. Pilot of MP-1 biofeedback rehabilitation in 5 patients; no questionnaire evaluated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Intervention study only</t>
+        </is>
+      </c>
+      <c r="S65" s="12" t="inlineStr">
+        <is>
+          <t>Pilot of MP-1 biofeedback rehabilitation in 5 patients; no questionnaire evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="9">
         <v>65</v>
       </c>
@@ -6662,13 +6916,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R66" s="12" t="inlineStr">
+      <c r="R66" s="12"/>
+      <c r="S66" s="12" t="inlineStr">
         <is>
           <t>Rasch evaluation of NEI VFQ-25 item functioning and sensitivity to change in veterans receiving LVR.</t>
         </is>
       </c>
     </row>
-    <row r="67" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="9">
         <v>66</v>
       </c>
@@ -6710,13 +6965,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R67" s="12" t="inlineStr">
+      <c r="R67" s="12"/>
+      <c r="S67" s="12" t="inlineStr">
         <is>
           <t>Validation (DIF, responsiveness) of the VA LV VFQ-48 in vision rehabilitation patients.</t>
         </is>
       </c>
     </row>
-    <row r="68" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="9">
         <v>67</v>
       </c>
@@ -6760,11 +7016,16 @@
       </c>
       <c r="R68" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Review/opinion/editorial. Narrative review of clinical reading tests; no questionnaire validation reported.</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Review/opinion/editorial</t>
+        </is>
+      </c>
+      <c r="S68" s="12" t="inlineStr">
+        <is>
+          <t>Narrative review of clinical reading tests; no questionnaire validation reported.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="9">
         <v>68</v>
       </c>
@@ -6810,11 +7071,16 @@
       </c>
       <c r="R69" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Intervention study only. MP-1 biofeedback rehabilitation in glaucoma; NEI VFQ-25 used only as an outcome, not validated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Intervention study only</t>
+        </is>
+      </c>
+      <c r="S69" s="12" t="inlineStr">
+        <is>
+          <t>MP-1 biofeedback rehabilitation in glaucoma; NEI VFQ-25 used only as an outcome, not validated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="9">
         <v>69</v>
       </c>
@@ -6860,11 +7126,16 @@
       </c>
       <c r="R70" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No accuracy/validation data. OCT vs visual function in multiple sclerosis; NEI VFQ collected but not evaluated as an instrument.</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No accuracy/validation data</t>
+        </is>
+      </c>
+      <c r="S70" s="12" t="inlineStr">
+        <is>
+          <t>OCT vs visual function in multiple sclerosis; NEI VFQ collected but not evaluated as an instrument.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="9">
         <v>70</v>
       </c>
@@ -6910,11 +7181,16 @@
       </c>
       <c r="R71" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No questionnaire/screening item. Population study linking objectively measured VI to dementia; no self-report vision tool evaluated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="S71" s="12" t="inlineStr">
+        <is>
+          <t>Population study linking objectively measured VI to dementia; no self-report vision tool evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="9">
         <v>71</v>
       </c>
@@ -6960,11 +7236,16 @@
       </c>
       <c r="R72" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Not about low vision/visual function. Pricing survey of specialists on off-label Avastin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Not about low vision/visual function</t>
+        </is>
+      </c>
+      <c r="S72" s="12" t="inlineStr">
+        <is>
+          <t>Pricing survey of specialists on off-label Avastin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="9">
         <v>72</v>
       </c>
@@ -7006,13 +7287,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R73" s="12" t="inlineStr">
+      <c r="R73" s="12"/>
+      <c r="S73" s="12" t="inlineStr">
         <is>
           <t>Compares responsiveness of IVI and NEI VFQ-25 in low vision patients after vision rehabilitation.</t>
         </is>
       </c>
     </row>
-    <row r="74" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="9">
         <v>73</v>
       </c>
@@ -7054,13 +7336,14 @@
           <t>Maybe</t>
         </is>
       </c>
-      <c r="R74" s="12" t="inlineStr">
+      <c r="R74" s="12"/>
+      <c r="S74" s="12" t="inlineStr">
         <is>
           <t>LVR outcome study using Rasch-scaled VA LV VFQ-48 and IVI; unclear whether any measurement-property data are reported.</t>
         </is>
       </c>
     </row>
-    <row r="75" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="9">
         <v>74</v>
       </c>
@@ -7102,13 +7385,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R75" s="12" t="inlineStr">
+      <c r="R75" s="12"/>
+      <c r="S75" s="12" t="inlineStr">
         <is>
           <t>Development and performance of the VA LV VFQ in low vision rehabilitation patients.</t>
         </is>
       </c>
     </row>
-    <row r="76" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="9">
         <v>75</v>
       </c>
@@ -7154,11 +7438,16 @@
       </c>
       <c r="R76" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No questionnaire/screening item. Fear-of-falling questionnaire (not a vision instrument) tested as a mediator of physical activity in glaucoma/AMD.</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="S76" s="12" t="inlineStr">
+        <is>
+          <t>Fear-of-falling questionnaire (not a vision instrument) tested as a mediator of physical activity in glaucoma/AMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="9">
         <v>76</v>
       </c>
@@ -7202,13 +7491,14 @@
           <t>Maybe</t>
         </is>
       </c>
-      <c r="R77" s="12" t="inlineStr">
+      <c r="R77" s="12"/>
+      <c r="S77" s="12" t="inlineStr">
         <is>
           <t>Examines construct validity of NEI VFQ-25 against a global QoL item; population and vision comparator unclear from abstract.</t>
         </is>
       </c>
     </row>
-    <row r="78" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="9">
         <v>77</v>
       </c>
@@ -7254,11 +7544,16 @@
       </c>
       <c r="R78" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Intervention study only. Biofeedback training in 6 AMD patients; questionnaire used only as an outcome.</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Intervention study only</t>
+        </is>
+      </c>
+      <c r="S78" s="12" t="inlineStr">
+        <is>
+          <t>Biofeedback training in 6 AMD patients; questionnaire used only as an outcome.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="9">
         <v>78</v>
       </c>
@@ -7304,11 +7599,16 @@
       </c>
       <c r="R79" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Review/opinion/editorial. Systematic review of Charles Bonnet syndrome prevalence; not about LVR screening questionnaires.</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Review/opinion/editorial</t>
+        </is>
+      </c>
+      <c r="S79" s="12" t="inlineStr">
+        <is>
+          <t>Systematic review of Charles Bonnet syndrome prevalence; not about LVR screening questionnaires.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="9">
         <v>79</v>
       </c>
@@ -7350,13 +7650,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R80" s="12" t="inlineStr">
+      <c r="R80" s="12"/>
+      <c r="S80" s="12" t="inlineStr">
         <is>
           <t>Two self-report screening questions (newsprint, face at 12 ft) assessed against examined VI with PPV/NPV in older adults.</t>
         </is>
       </c>
     </row>
-    <row r="81" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="9">
         <v>80</v>
       </c>
@@ -7402,11 +7703,16 @@
       </c>
       <c r="R81" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No accuracy/validation data. Population prevalence study of myopic macular degeneration; VF-11 questionnaire used only as an outcome, not evaluated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No accuracy/validation data</t>
+        </is>
+      </c>
+      <c r="S81" s="12" t="inlineStr">
+        <is>
+          <t>Population prevalence study of myopic macular degeneration; VF-11 questionnaire used only as an outcome, not evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="9">
         <v>81</v>
       </c>
@@ -7452,11 +7758,16 @@
       </c>
       <c r="R82" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Wrong population (not adults). Screening tool for cerebral visual impairment in children aged 3-50 months.</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Wrong population (not adults)</t>
+        </is>
+      </c>
+      <c r="S82" s="12" t="inlineStr">
+        <is>
+          <t>Screening tool for cerebral visual impairment in children aged 3-50 months.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="9">
         <v>82</v>
       </c>
@@ -7502,11 +7813,16 @@
       </c>
       <c r="R83" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Review/opinion/editorial. Narrative overview of LVR service principles; no questionnaire data and not a referral guideline.</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Review/opinion/editorial</t>
+        </is>
+      </c>
+      <c r="S83" s="12" t="inlineStr">
+        <is>
+          <t>Narrative overview of LVR service principles; no questionnaire data and not a referral guideline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="9">
         <v>83</v>
       </c>
@@ -7552,11 +7868,16 @@
       </c>
       <c r="R84" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No questionnaire/screening item. Halo software test of visual discrimination in drivers; driving questionnaire not evaluated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="S84" s="12" t="inlineStr">
+        <is>
+          <t>Halo software test of visual discrimination in drivers; driving questionnaire not evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="9">
         <v>84</v>
       </c>
@@ -7598,13 +7919,14 @@
           <t>Maybe</t>
         </is>
       </c>
-      <c r="R85" s="12" t="inlineStr">
+      <c r="R85" s="12"/>
+      <c r="S85" s="12" t="inlineStr">
         <is>
           <t>NEI VFQ-25 correlated with measured visual function in Stargardt disease; small sample, and adult age needs confirming.</t>
         </is>
       </c>
     </row>
-    <row r="86" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="9">
         <v>85</v>
       </c>
@@ -7648,13 +7970,14 @@
           <t>Maybe</t>
         </is>
       </c>
-      <c r="R86" s="12" t="inlineStr">
+      <c r="R86" s="12"/>
+      <c r="S86" s="12" t="inlineStr">
         <is>
           <t>Qualitative content-validity refinement of an LVR outcome instrument (LVIM); no psychometric data, but relevant to LVR tools.</t>
         </is>
       </c>
     </row>
-    <row r="87" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="9">
         <v>86</v>
       </c>
@@ -7696,13 +8019,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R87" s="12" t="inlineStr">
+      <c r="R87" s="12"/>
+      <c r="S87" s="12" t="inlineStr">
         <is>
           <t>Rasch-analysed Participation and Activity Inventory measuring rehabilitative need in adults entering LVR, related to VA and other measures.</t>
         </is>
       </c>
     </row>
-    <row r="88" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="9">
         <v>87</v>
       </c>
@@ -7748,11 +8072,16 @@
       </c>
       <c r="R88" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No accuracy/validation data. Population study of vision and fear of falling; single self-rated vision item used as exposure, not validated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No accuracy/validation data</t>
+        </is>
+      </c>
+      <c r="S88" s="12" t="inlineStr">
+        <is>
+          <t>Population study of vision and fear of falling; single self-rated vision item used as exposure, not validated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="9">
         <v>88</v>
       </c>
@@ -7796,13 +8125,14 @@
           <t>Maybe</t>
         </is>
       </c>
-      <c r="R89" s="12" t="inlineStr">
+      <c r="R89" s="12"/>
+      <c r="S89" s="12" t="inlineStr">
         <is>
           <t>Responsiveness and discrimination of the generic EQ-5D tested against the Activity Inventory in LVR patients; measurement-property data, but EQ-5D is not a vision-specific instrument.</t>
         </is>
       </c>
     </row>
-    <row r="90" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="9">
         <v>89</v>
       </c>
@@ -7844,13 +8174,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R90" s="12" t="inlineStr">
+      <c r="R90" s="12"/>
+      <c r="S90" s="12" t="inlineStr">
         <is>
           <t>Rasch-based responsiveness validation of the LVIM-R in adults receiving low vision rehabilitation.</t>
         </is>
       </c>
     </row>
-    <row r="91" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="9">
         <v>90</v>
       </c>
@@ -7896,11 +8227,16 @@
       </c>
       <c r="R91" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No questionnaire/screening item. Falls and injuries in AMD predicted by clinical vision measures; no self-report tool evaluated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="S91" s="12" t="inlineStr">
+        <is>
+          <t>Falls and injuries in AMD predicted by clinical vision measures; no self-report tool evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="9">
         <v>91</v>
       </c>
@@ -7946,11 +8282,16 @@
       </c>
       <c r="R92" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No questionnaire/screening item. Two-participant study of BCI/eye-tracking typing in ALS; no questionnaire evaluated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="S92" s="12" t="inlineStr">
+        <is>
+          <t>Two-participant study of BCI/eye-tracking typing in ALS; no questionnaire evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="9">
         <v>92</v>
       </c>
@@ -7992,13 +8333,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R93" s="12" t="inlineStr">
+      <c r="R93" s="12"/>
+      <c r="S93" s="12" t="inlineStr">
         <is>
           <t>Screening questions (menu, keyboard) vs measured VA in 385 adults with sensitivity, specificity and AUC; core study.</t>
         </is>
       </c>
     </row>
-    <row r="94" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="9">
         <v>93</v>
       </c>
@@ -8038,13 +8380,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R94" s="12" t="inlineStr">
+      <c r="R94" s="12"/>
+      <c r="S94" s="12" t="inlineStr">
         <is>
           <t>USPSTF systematic review that summarises accuracy of screening questions vs VA testing in older adults.</t>
         </is>
       </c>
     </row>
-    <row r="95" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="9">
         <v>94</v>
       </c>
@@ -8090,11 +8433,16 @@
       </c>
       <c r="R95" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Wrong population (not adults). Parent-reported CVI questionnaire in children.</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Wrong population (not adults)</t>
+        </is>
+      </c>
+      <c r="S95" s="12" t="inlineStr">
+        <is>
+          <t>Parent-reported CVI questionnaire in children.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="9">
         <v>95</v>
       </c>
@@ -8138,13 +8486,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R96" s="12" t="inlineStr">
+      <c r="R96" s="12"/>
+      <c r="S96" s="12" t="inlineStr">
         <is>
           <t>Rasch validation of self-reported driving difficulty in 851 low-vision clinic patients, related to VA and CS.</t>
         </is>
       </c>
     </row>
-    <row r="97" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="9">
         <v>96</v>
       </c>
@@ -8190,11 +8539,16 @@
       </c>
       <c r="R97" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Intervention study only. PRL biofeedback training outcomes; VFQ-25 used only as an outcome measure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="98" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Intervention study only</t>
+        </is>
+      </c>
+      <c r="S97" s="12" t="inlineStr">
+        <is>
+          <t>PRL biofeedback training outcomes; VFQ-25 used only as an outcome measure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="9">
         <v>97</v>
       </c>
@@ -8238,13 +8592,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R98" s="12" t="inlineStr">
+      <c r="R98" s="12"/>
+      <c r="S98" s="12" t="inlineStr">
         <is>
           <t>Develops and Rasch-validates the Spatial Localization Questionnaire against clinical vision tests in visually impaired adults.</t>
         </is>
       </c>
     </row>
-    <row r="99" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="9">
         <v>98</v>
       </c>
@@ -8290,11 +8645,16 @@
       </c>
       <c r="R99" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No accuracy/validation data. Driving simulator speed study in cataract; Driver Habits Questionnaire used descriptively without validation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No accuracy/validation data</t>
+        </is>
+      </c>
+      <c r="S99" s="12" t="inlineStr">
+        <is>
+          <t>Driving simulator speed study in cataract; Driver Habits Questionnaire used descriptively without validation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="9">
         <v>99</v>
       </c>
@@ -8340,11 +8700,16 @@
       </c>
       <c r="R100" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Intervention study only. RCT and cost-effectiveness of basic LVR; no questionnaire validation or screening data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Intervention study only</t>
+        </is>
+      </c>
+      <c r="S100" s="12" t="inlineStr">
+        <is>
+          <t>RCT and cost-effectiveness of basic LVR; no questionnaire validation or screening data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="9">
         <v>100</v>
       </c>
@@ -8390,11 +8755,16 @@
       </c>
       <c r="R101" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No accuracy/validation data. Self-reported VI (NEI-VFQ) as an exposure for cognitive decline; no validation against vision.</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No accuracy/validation data</t>
+        </is>
+      </c>
+      <c r="S101" s="12" t="inlineStr">
+        <is>
+          <t>Self-reported VI (NEI-VFQ) as an exposure for cognitive decline; no validation against vision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="9">
         <v>101</v>
       </c>
@@ -8440,11 +8810,16 @@
       </c>
       <c r="R102" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Intervention study only. Head-mounted device trial; VA LV VFQ-48 used only as an outcome measure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="103" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Intervention study only</t>
+        </is>
+      </c>
+      <c r="S102" s="12" t="inlineStr">
+        <is>
+          <t>Head-mounted device trial; VA LV VFQ-48 used only as an outcome measure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="9">
         <v>102</v>
       </c>
@@ -8490,11 +8865,16 @@
       </c>
       <c r="R103" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Wrong population (not adults). CVI diagnosis and referral guidelines for children aged 18 or under.</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Wrong population (not adults)</t>
+        </is>
+      </c>
+      <c r="S103" s="12" t="inlineStr">
+        <is>
+          <t>CVI diagnosis and referral guidelines for children aged 18 or under.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="9">
         <v>103</v>
       </c>
@@ -8540,11 +8920,16 @@
       </c>
       <c r="R104" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No questionnaire/screening item. Home hazards, measured vision and falls; no self-report vision tool evaluated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="S104" s="12" t="inlineStr">
+        <is>
+          <t>Home hazards, measured vision and falls; no self-report vision tool evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="9">
         <v>104</v>
       </c>
@@ -8590,11 +8975,16 @@
       </c>
       <c r="R105" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No questionnaire/screening item. Season, sunlight and depressive symptoms in VI; no vision self-report tool evaluated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="S105" s="12" t="inlineStr">
+        <is>
+          <t>Season, sunlight and depressive symptoms in VI; no vision self-report tool evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="9">
         <v>105</v>
       </c>
@@ -8636,13 +9026,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R106" s="12" t="inlineStr">
+      <c r="R106" s="12"/>
+      <c r="S106" s="12" t="inlineStr">
         <is>
           <t>Validation of the Italian VA LV VFQ-48 in LVR patients, with reliability and correlation with VA and reading.</t>
         </is>
       </c>
     </row>
-    <row r="107" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="9">
         <v>106</v>
       </c>
@@ -8688,11 +9079,16 @@
       </c>
       <c r="R107" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No accuracy/validation data. Gaze perception task study; brief questionnaire used as a predictor, not validated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No accuracy/validation data</t>
+        </is>
+      </c>
+      <c r="S107" s="12" t="inlineStr">
+        <is>
+          <t>Gaze perception task study; brief questionnaire used as a predictor, not validated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="9">
         <v>107</v>
       </c>
@@ -8738,11 +9134,16 @@
       </c>
       <c r="R108" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No accuracy/validation data. Determinants-of-QoL regression in LV clinic patients; questionnaires used as outcomes, not validated or tested for accuracy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="109" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No accuracy/validation data</t>
+        </is>
+      </c>
+      <c r="S108" s="12" t="inlineStr">
+        <is>
+          <t>Determinants-of-QoL regression in LV clinic patients; questionnaires used as outcomes, not validated or tested for accuracy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="9">
         <v>108</v>
       </c>
@@ -8784,13 +9185,14 @@
           <t>Maybe</t>
         </is>
       </c>
-      <c r="R109" s="12" t="inlineStr">
+      <c r="R109" s="12"/>
+      <c r="S109" s="12" t="inlineStr">
         <is>
           <t>Population study relating NEI VFQ-25 scores to measured acuity and eye disease incl. glaucoma; may give known-groups validity data for a full-length questionnaire.</t>
         </is>
       </c>
     </row>
-    <row r="110" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="9">
         <v>109</v>
       </c>
@@ -8836,11 +9238,16 @@
       </c>
       <c r="R110" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No questionnaire/screening item. Work ability and psychosocial work questionnaires in low vision; no vision self-report tool evaluated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="S110" s="12" t="inlineStr">
+        <is>
+          <t>Work ability and psychosocial work questionnaires in low vision; no vision self-report tool evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="9">
         <v>110</v>
       </c>
@@ -8882,13 +9289,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R111" s="12" t="inlineStr">
+      <c r="R111" s="12"/>
+      <c r="S111" s="12" t="inlineStr">
         <is>
           <t>Glaucoma patients' visual disability questionnaire correlated against Humphrey VF and VA (glaucoma PROM vs measured vision).</t>
         </is>
       </c>
     </row>
-    <row r="112" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="9">
         <v>111</v>
       </c>
@@ -8934,11 +9342,16 @@
       </c>
       <c r="R112" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No questionnaire/screening item. Falls vs visual function in low vision; ADL questionnaire only a covariate, not evaluated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="113" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="S112" s="12" t="inlineStr">
+        <is>
+          <t>Falls vs visual function in low vision; ADL questionnaire only a covariate, not evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="9">
         <v>112</v>
       </c>
@@ -8980,13 +9393,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R113" s="12" t="inlineStr">
+      <c r="R113" s="12"/>
+      <c r="S113" s="12" t="inlineStr">
         <is>
           <t>Adults &gt;50 in primary care; compares time to administer the Functional Vision Screening Questionnaire with chart tests (feasibility outcome in PICO).</t>
         </is>
       </c>
     </row>
-    <row r="114" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="9">
         <v>113</v>
       </c>
@@ -9032,11 +9446,16 @@
       </c>
       <c r="R114" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Wrong population (not adults). Parent-reported CVI screening questionnaires in children.</t>
-        </is>
-      </c>
-    </row>
-    <row r="115" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Wrong population (not adults)</t>
+        </is>
+      </c>
+      <c r="S114" s="12" t="inlineStr">
+        <is>
+          <t>Parent-reported CVI screening questionnaires in children.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="9">
         <v>114</v>
       </c>
@@ -9080,13 +9499,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R115" s="12" t="inlineStr">
+      <c r="R115" s="12"/>
+      <c r="S115" s="12" t="inlineStr">
         <is>
           <t>Psychometric validation (reliability, known-groups by VA) of Thai vision bolt-on EQ-5D in visually impaired participants.</t>
         </is>
       </c>
     </row>
-    <row r="116" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="9">
         <v>115</v>
       </c>
@@ -9132,11 +9552,16 @@
       </c>
       <c r="R116" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No accuracy/validation data. Translation and cultural adaptation of LVQOL only; psychometric validation deferred to a later study.</t>
-        </is>
-      </c>
-    </row>
-    <row r="117" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No accuracy/validation data</t>
+        </is>
+      </c>
+      <c r="S116" s="12" t="inlineStr">
+        <is>
+          <t>Translation and cultural adaptation of LVQOL only; psychometric validation deferred to a later study.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="9">
         <v>116</v>
       </c>
@@ -9182,11 +9607,16 @@
       </c>
       <c r="R117" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No questionnaire/screening item. Cohort study of measured VA and mortality; no self-report tool.</t>
-        </is>
-      </c>
-    </row>
-    <row r="118" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="S117" s="12" t="inlineStr">
+        <is>
+          <t>Cohort study of measured VA and mortality; no self-report tool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="9">
         <v>117</v>
       </c>
@@ -9230,11 +9660,16 @@
       </c>
       <c r="R118" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Not about low vision/visual function. Symptom questionnaire to differentiate dry eye from other diagnoses; not judged against vision impairment or LVR need.</t>
-        </is>
-      </c>
-    </row>
-    <row r="119" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Not about low vision/visual function</t>
+        </is>
+      </c>
+      <c r="S118" s="12" t="inlineStr">
+        <is>
+          <t>Symptom questionnaire to differentiate dry eye from other diagnoses; not judged against vision impairment or LVR need.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="9">
         <v>118</v>
       </c>
@@ -9280,11 +9715,16 @@
       </c>
       <c r="R119" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Wrong population (not adults). Validation of an iPad CVI screening app in children aged 5-18.</t>
-        </is>
-      </c>
-    </row>
-    <row r="120" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Wrong population (not adults)</t>
+        </is>
+      </c>
+      <c r="S119" s="12" t="inlineStr">
+        <is>
+          <t>Validation of an iPad CVI screening app in children aged 5-18.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="9">
         <v>119</v>
       </c>
@@ -9326,13 +9766,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R120" s="12" t="inlineStr">
+      <c r="R120" s="12"/>
+      <c r="S120" s="12" t="inlineStr">
         <is>
           <t>Validation of Spanish LVQOL with reliability, IRT and sensitivity/specificity cut-off for detecting visual impairment.</t>
         </is>
       </c>
     </row>
-    <row r="121" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="9">
         <v>120</v>
       </c>
@@ -9374,13 +9815,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R121" s="12" t="inlineStr">
+      <c r="R121" s="12"/>
+      <c r="S121" s="12" t="inlineStr">
         <is>
           <t>Self-reported mobility questionnaire validated against VA, CS and VF in low vision patients, proposed as guide for O&amp;M referral.</t>
         </is>
       </c>
     </row>
-    <row r="122" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="9">
         <v>121</v>
       </c>
@@ -9422,13 +9864,14 @@
           <t>Maybe</t>
         </is>
       </c>
-      <c r="R122" s="12" t="inlineStr">
+      <c r="R122" s="12"/>
+      <c r="S122" s="12" t="inlineStr">
         <is>
           <t>Visual difficulty questionnaire with factor and discriminant analysis between low-vision and nonimpaired older drivers; unclear if accuracy data reported.</t>
         </is>
       </c>
     </row>
-    <row r="123" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="9">
         <v>122</v>
       </c>
@@ -9470,13 +9913,14 @@
           <t>Include</t>
         </is>
       </c>
-      <c r="R123" s="12" t="inlineStr">
+      <c r="R123" s="12"/>
+      <c r="S123" s="12" t="inlineStr">
         <is>
           <t>LVQOL in advanced glaucoma with low vision related to VA, MD and edge detection with AUROC analysis (glaucoma PROM study).</t>
         </is>
       </c>
     </row>
-    <row r="124" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="9">
         <v>123</v>
       </c>
@@ -9522,11 +9966,16 @@
       </c>
       <c r="R124" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No questionnaire/screening item. Postural sway vs visual field loss in glaucoma; no self-report vision tool evaluated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="125" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="S124" s="12" t="inlineStr">
+        <is>
+          <t>Postural sway vs visual field loss in glaucoma; no self-report vision tool evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="9">
         <v>124</v>
       </c>
@@ -9572,11 +10021,16 @@
       </c>
       <c r="R125" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No accuracy/validation data. Self-reported VFQ used only as a predictor of physical performance decline; not validated against vision measures.</t>
-        </is>
-      </c>
-    </row>
-    <row r="126" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No accuracy/validation data</t>
+        </is>
+      </c>
+      <c r="S125" s="12" t="inlineStr">
+        <is>
+          <t>Self-reported VFQ used only as a predictor of physical performance decline; not validated against vision measures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="9">
         <v>125</v>
       </c>
@@ -9622,11 +10076,16 @@
       </c>
       <c r="R126" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No accuracy/validation data. Self-reported visual difficulty used as an exposure for sleep outcomes; no accuracy or validation of the item.</t>
-        </is>
-      </c>
-    </row>
-    <row r="127" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>No accuracy/validation data</t>
+        </is>
+      </c>
+      <c r="S126" s="12" t="inlineStr">
+        <is>
+          <t>Self-reported visual difficulty used as an exposure for sleep outcomes; no accuracy or validation of the item.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="9">
         <v>126</v>
       </c>
@@ -9672,11 +10131,16 @@
       </c>
       <c r="R127" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: Not about low vision/visual function. Self-assessed driving skill vs on-road evaluation in bioptic drivers; not a vision/LVR-need screening tool.</t>
-        </is>
-      </c>
-    </row>
-    <row r="128" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+          <t>Not about low vision/visual function</t>
+        </is>
+      </c>
+      <c r="S127" s="12" t="inlineStr">
+        <is>
+          <t>Self-assessed driving skill vs on-road evaluation in bioptic drivers; not a vision/LVR-need screening tool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="9">
         <v>127</v>
       </c>
@@ -9722,12 +10186,17 @@
       </c>
       <c r="R128" s="12" t="inlineStr">
         <is>
-          <t>Exclusion reason: No questionnaire/screening item. Survey of orthoptists' LVR practice for AMD in France; no patient self-report tool or referral guideline.</t>
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="S128" s="12" t="inlineStr">
+        <is>
+          <t>Survey of orthoptists' LVR practice for AMD in France; no patient self-report tool or referral guideline.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R128" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:S128" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <conditionalFormatting sqref="H2:H128">
     <cfRule type="expression" dxfId="8" priority="2">
       <formula>H2="Include"</formula>

</xml_diff>

<commit_message>
Add the eight hand-added key sources to the screening workbook
Add records 128-135, the key sources from data/LVR_Q_Study_Outline.md
that the PubMed and Scopus searches missed, to the Screening tab as
rows 129-136. The reviewer columns are blank, ready for screening,
and there is no Zotero key or AI suggestion yet.

On the Counts tab, add "Records identified - other sources" (8), which
brings the total identified to 174 and records screened to 135, and
extend the formula ranges to row 136. Regenerate the Screening and
Counts CSVs.

Update CLAUDE.md for the new record range, and warn against saving
the source workbook with openpyxl, which deletes its x14 drop-downs.
Update AI_strict_screening_rules.md, which said these records were
not in the workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/LVR_screening_sheet_2.xlsx
+++ b/data/LVR_screening_sheet_2.xlsx
@@ -19,7 +19,7 @@
     <sheet name="Lists" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Screening!$A$1:$P$128</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Screening!$A$1:$P$136</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -3243,7 +3243,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:S128"/>
+  <dimension ref="A1:S136"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -10195,9 +10195,353 @@
         </is>
       </c>
     </row>
+    <row r="129" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A129" s="9">
+        <v>128</v>
+      </c>
+      <c r="B129" s="9">
+        <v>2024</v>
+      </c>
+      <c r="C129" s="9" t="inlineStr">
+        <is>
+          <t>Wu, Yueh-Hsun et al.</t>
+        </is>
+      </c>
+      <c r="D129" s="9" t="inlineStr">
+        <is>
+          <t>Estimating Visual Acuity Without a Visual Acuity Chart.</t>
+        </is>
+      </c>
+      <c r="E129" s="9" t="inlineStr">
+        <is>
+          <t>Translational vision science &amp; technology</t>
+        </is>
+      </c>
+      <c r="F129" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="G129" s="9" t="inlineStr">
+        <is>
+          <t>PURPOSE: This study explored whether visual acuity (VA) can be inferred from self-reported ability to recognize everyday objects using a set of yes/no questions. METHODS: Participants answered 100 yes/no questions designed to assess their ability to recognize familiar objects at typical viewing distances, such as distinguishing between a full moon and a half moon on a clear night. The questions demanded VA ranging from normal to severe vision impairment. Responses were analyzed using item response theory, and the results were compared with participants' VA values. RESULTS: We recruited 385 participants from 4 sites in the United States. Participants had a mean age of 56.7 years with VA ranging from -0.3 to 2.0 logarithm of the minimum angle of resolution (logMAR) (mean = 0.58). A strong relationship was observed between participants' estimated vision ability and their VA (r = -0.72). The linear relationship can be used to predict each participant's VA based on their estimated vision ability. The average signed and unsigned prediction errors were 0 and 0.24 logMAR, respectively, with a coefficient of repeatability of 0.59 logMAR between the estimated VA and measured VA. The same linear function was used to determine the VA limit required for each question. For instance, the VA limit for the moon question was 1.0 logMAR. CONCLUSIONS: Yes/no questions about everyday visual activities have the potential to estimate an individual's VA. Future refinements may enhance reliability. TRANSLATIONAL RELEVANCE: The survey provides insights into the real-world visual capabilities of people with low vision, making it potentially useful for telehealth applications.</t>
+        </is>
+      </c>
+      <c r="H129" s="11"/>
+      <c r="I129" s="11"/>
+      <c r="J129" s="11"/>
+      <c r="K129" s="11"/>
+      <c r="L129" s="11"/>
+      <c r="M129" s="9"/>
+      <c r="N129" s="12"/>
+      <c r="O129" s="12"/>
+      <c r="P129" s="12"/>
+      <c r="Q129" s="12"/>
+      <c r="R129" s="12"/>
+      <c r="S129" s="12"/>
+    </row>
+    <row r="130" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A130" s="9">
+        <v>129</v>
+      </c>
+      <c r="B130" s="9">
+        <v>2023</v>
+      </c>
+      <c r="C130" s="9" t="inlineStr">
+        <is>
+          <t>Vinokurtseva, Anastasiya et al.</t>
+        </is>
+      </c>
+      <c r="D130" s="9" t="inlineStr">
+        <is>
+          <t>Evaluating Measurement Properties of Patient-Reported Outcome Measures in Glaucoma: A Systematic Review.</t>
+        </is>
+      </c>
+      <c r="E130" s="9" t="inlineStr">
+        <is>
+          <t>Ophthalmology. Glaucoma</t>
+        </is>
+      </c>
+      <c r="F130" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="G130" s="9" t="inlineStr">
+        <is>
+          <t>TOPIC: The purpose of the current study was to systematically identify and evaluate existing patient-reported outcome measures (PROMs) for clinical glaucoma practice. CLINICAL RELEVANCE: Understanding and incorporating patient preferences into decision-making is now recognized as critical for optimal resource allocation, especially in technologically advancing areas, such as minimally invasive surgeries. Patient-reported outcome measures are instruments designed to evaluate the health outcomes that are most important to patients. Despite their recognized importance, especially in the era of patient-centered care, their routine use in clinical settings remains low. METHODS: A systematic literature search was conducted in 6 databases (EMBASE, MEDLINE, PsycINFO, Scopus, BIOSIS, and Web of Science) from the date of inception. Studies were included in the qualitative review if they reported measurement properties of PROMs in adult patients with glaucoma. COnsensus-based Standards for the selection of health Measurement INstruments guidelines were used to assess the included PROMs. The study protocol is registered with PROSPERO (registration number: CRD42020176064). RESULTS: The literature search yielded 2661 records. After deduplication, 1259 studies entered level 1 screening, and based on title and abstract review, 164 records proceeded to full-text screening. In 48 included studies, 70 instrument reports discuss 43 distinct instruments in 3 major categories: glaucoma-specific, vision-specific, and general health-related quality of life. Most used measures were glaucoma-specific (Glaucoma Quality of Life [GQL] and Glaucoma Symptom Scale [GSS]) and vision-specific (National Eye Institute Visual Function Questionnaire [NEI VFQ-25]). All 3 have sufficient validity (especially construct), with GQL and GSS having sufficient internal consistency, cross-cultural validity, and reliability, with reports suggesting high methodological quality. CONCLUSION: The GQL, GSS, and NEI VFQ-25 are the 3 most used questionnaires in a research setting, having considerable validation in a patient population with glaucoma. Limited reports on interpretability, responsiveness, and feasibility in all 43 identified instruments make identifying a single optimal questionnaire for clinical use challenging and highlight the need for further studies. FINANCIAL DISCLOSURE(S): Proprietary or commercial disclosure may be found in the Footnotes and Disclosures at the end of this article.</t>
+        </is>
+      </c>
+      <c r="H130" s="11"/>
+      <c r="I130" s="11"/>
+      <c r="J130" s="11"/>
+      <c r="K130" s="11"/>
+      <c r="L130" s="11"/>
+      <c r="M130" s="9"/>
+      <c r="N130" s="12"/>
+      <c r="O130" s="12"/>
+      <c r="P130" s="12"/>
+      <c r="Q130" s="12"/>
+      <c r="R130" s="12"/>
+      <c r="S130" s="12"/>
+    </row>
+    <row r="131" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A131" s="9">
+        <v>130</v>
+      </c>
+      <c r="B131" s="9">
+        <v>2025</v>
+      </c>
+      <c r="C131" s="9" t="inlineStr">
+        <is>
+          <t>Ernst, Julia et al.</t>
+        </is>
+      </c>
+      <c r="D131" s="9" t="inlineStr">
+        <is>
+          <t>Factors Associated with Referral to Low Vision for Patients with Advanced Glaucoma.</t>
+        </is>
+      </c>
+      <c r="E131" s="9" t="inlineStr">
+        <is>
+          <t>Life (Basel, Switzerland)</t>
+        </is>
+      </c>
+      <c r="F131" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="G131" s="9" t="inlineStr">
+        <is>
+          <t>Glaucoma is one of the most common causes of irreversible visual impairment world wide. Providing low vision rehabilitation (LVR) services is a primary mode of support for patients with permanent vision loss. This retrospective, cross-sectional study evaluated the rate at which patients with severe open-angle glaucoma (OAG) were referred for LVR services at an academic medical center. Patient demographics, glaucoma severity, appointment history, performance on visual field (VF) testing, presenting visual acuity (VA), and change in best-corrected visual acuity (BCVA) after low vision refraction were abstracted from the electronic record and summarized by using descriptive statistics. Logistic regression analysis was used to assess the relationship between study variables and the likelihood of referral for LVR evaluation. Out of 522 patients with severe OAG, 88% of whom qualified as having low vision, 14 were referred for an LVR evaluation (2.7%). Referrals were most strongly associated with VA (adjusted odds ratio [aOR], 7.20; 95% confidence interval [CI], 2.11-24.64, p = 0.001) but not glaucoma-associated VF loss (aOR, 0.90; 95% CI, 0.24-3.37, p = 0.876). Thirteen of 14 patients referred for LVR completed visits (93%). More than one-third of those patients improved in their better-seeing eye after a low vision refraction, gaining an average of -0.18 ± 0.24 logMAR (half gaining ≥2-lines of BCVA). Patients with severe OAG are at risk of progressive visual disability from their eye disease. We found, however, that the majority of these patients were not referred to LVR services, despite meeting eligibility criteria and growing evidence demonstrating their potential benefit.</t>
+        </is>
+      </c>
+      <c r="H131" s="11"/>
+      <c r="I131" s="11"/>
+      <c r="J131" s="11"/>
+      <c r="K131" s="11"/>
+      <c r="L131" s="11"/>
+      <c r="M131" s="9"/>
+      <c r="N131" s="12"/>
+      <c r="O131" s="12"/>
+      <c r="P131" s="12"/>
+      <c r="Q131" s="12"/>
+      <c r="R131" s="12"/>
+      <c r="S131" s="12"/>
+    </row>
+    <row r="132" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A132" s="9">
+        <v>131</v>
+      </c>
+      <c r="B132" s="9">
+        <v>2017</v>
+      </c>
+      <c r="C132" s="9" t="inlineStr">
+        <is>
+          <t>Swenor, Bonnielin K et al.</t>
+        </is>
+      </c>
+      <c r="D132" s="9" t="inlineStr">
+        <is>
+          <t>Impact of the Ability to Divide Attention on Reading Performance in Glaucoma.</t>
+        </is>
+      </c>
+      <c r="E132" s="9" t="inlineStr">
+        <is>
+          <t>Investigative ophthalmology &amp; visual science</t>
+        </is>
+      </c>
+      <c r="F132" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="G132" s="9" t="inlineStr">
+        <is>
+          <t>PURPOSE: To determine if the ability to divide attention affects the relationship between glaucoma-related vision loss and reading speed. METHODS: Better eye mean deviation (MD), contrast sensitivity (CS), and better-eye distance visual acuity (VA) were measured in 28 participants with glaucoma and 21 controls. Reading speeds were assessed using MNRead, IRest, and sustained silent reading tests (words per minute, wpm). The ability to divide attention was measured using the Brief Test of Attention (BTA; scored 0-10). Multivariable linear regression models were used to determine the relationship between visual factors and reading speeds. Effect modification by BTA score (low BTA: &lt;7; high BTA: ≥7) was examined. RESULTS: Worse CS (per 0.1 log unit) was associated with slower maximum reading speed on MNRead test for participants with low BTA scores (β = -9 wpm; 95% confidence interval [CI]: -16, -2), but not for those with high BTA scores (β = -2 wpm; 95% CI: -6, +2). Similarly, for the IRest test, worse CS was associated with slower reading speeds (β = -12 wpm; 95% CI: -20, -4) among those with low, but not high BTA scores (β = -4 wpm; 95% CI: -10, +2). For the sustained silent reading test, glaucoma status (versus controls), worse visual field (VF) MD (per 5 dB), and worse CS were associated with 39%, 21%, and 19% slower reading speeds, respectively, for those with low BTA scores (P &lt; 0.05), but these associations were not significant among those with high BTA scores (P &gt; 0.1 for all). CONCLUSIONS: Decreased ability to divide attention, indicated by lower BTA scores, is associated with slower reading speeds in glaucoma with reduced CS and VF defects.</t>
+        </is>
+      </c>
+      <c r="H132" s="11"/>
+      <c r="I132" s="11"/>
+      <c r="J132" s="11"/>
+      <c r="K132" s="11"/>
+      <c r="L132" s="11"/>
+      <c r="M132" s="9"/>
+      <c r="N132" s="12"/>
+      <c r="O132" s="12"/>
+      <c r="P132" s="12"/>
+      <c r="Q132" s="12"/>
+      <c r="R132" s="12"/>
+      <c r="S132" s="12"/>
+    </row>
+    <row r="133" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A133" s="9">
+        <v>132</v>
+      </c>
+      <c r="B133" s="9">
+        <v>2022</v>
+      </c>
+      <c r="C133" s="9" t="inlineStr">
+        <is>
+          <t>Healthwise Staff</t>
+        </is>
+      </c>
+      <c r="D133" s="9" t="inlineStr">
+        <is>
+          <t>Legal blindness</t>
+        </is>
+      </c>
+      <c r="E133" s="9" t="inlineStr">
+        <is>
+          <t>HealthLink BC (website)</t>
+        </is>
+      </c>
+      <c r="F133" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="G133" s="9" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="H133" s="11"/>
+      <c r="I133" s="11"/>
+      <c r="J133" s="11"/>
+      <c r="K133" s="11"/>
+      <c r="L133" s="11"/>
+      <c r="M133" s="9"/>
+      <c r="N133" s="12"/>
+      <c r="O133" s="12"/>
+      <c r="P133" s="12"/>
+      <c r="Q133" s="12"/>
+      <c r="R133" s="12"/>
+      <c r="S133" s="12"/>
+    </row>
+    <row r="134" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A134" s="9">
+        <v>133</v>
+      </c>
+      <c r="B134" s="9">
+        <v>2014</v>
+      </c>
+      <c r="C134" s="9" t="inlineStr">
+        <is>
+          <t>Nguyen, Angeline M et al.</t>
+        </is>
+      </c>
+      <c r="D134" s="9" t="inlineStr">
+        <is>
+          <t>Reading ability and reading engagement in older adults with glaucoma.</t>
+        </is>
+      </c>
+      <c r="E134" s="9" t="inlineStr">
+        <is>
+          <t>Investigative ophthalmology &amp; visual science</t>
+        </is>
+      </c>
+      <c r="F134" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="G134" s="9" t="inlineStr">
+        <is>
+          <t>PURPOSE: We evaluated the impact of glaucoma-related vision loss on reading ability and reading engagement in 10 reading activities. METHODS: A total of 63 glaucoma patients and 59 glaucoma suspect controls self-rated their level of reading difficulty for 10 reading items, and responses were analyzed using Rasch analysis to determine reading ability. Reading engagement was assessed by asking subjects to report the number of days per week they engaged in each reading activity. Reading restriction was determined as a decrement in engagement. RESULTS: Glaucoma subjects more often described greater reading difficulty than controls for all tasks except puzzles (P &lt; 0.05). The most difficult reading tasks involved puzzles, books, and finances, while the least difficult reading tasks involved notes, bills, and mail. In multivariable weighted least squares regression models of Rasch-estimated person measures of reading ability, less reading ability was found for glaucoma patients compared to controls (β = -1.60 logits, P &lt; 0.001). Among glaucoma patients, less reading ability was associated with more severe visual field (VF) loss (β = -0.68 logits per 5-dB decrement in better-eye VF mean deviation [MD], P &lt; 0.001) and contrast sensitivity (β = -0.76 logits per 0.1-unit lower log CS, P &lt; 0.001). Each 5-dB decrement in the better-eye VF MD was associated with book reading on 18% fewer days (P = 0.003) and newspaper reading on 10% fewer days (P = 0.008). No statistically significant reading restriction was observed for other reading activities (P &gt; 0.05). CONCLUSIONS: Glaucoma patients have less reading ability and engage less in a variety of different reading activities, particularly those requiring sustained reading. Future work should evaluate the mechanisms underlying reading disability in glaucoma to determine how patients can maintain reading ability and engagement.</t>
+        </is>
+      </c>
+      <c r="H134" s="11"/>
+      <c r="I134" s="11"/>
+      <c r="J134" s="11"/>
+      <c r="K134" s="11"/>
+      <c r="L134" s="11"/>
+      <c r="M134" s="9"/>
+      <c r="N134" s="12"/>
+      <c r="O134" s="12"/>
+      <c r="P134" s="12"/>
+      <c r="Q134" s="12"/>
+      <c r="R134" s="12"/>
+      <c r="S134" s="12"/>
+    </row>
+    <row r="135" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A135" s="9">
+        <v>134</v>
+      </c>
+      <c r="B135" s="9">
+        <v>2017</v>
+      </c>
+      <c r="C135" s="9" t="inlineStr">
+        <is>
+          <t>Kaleem, Mona A et al.</t>
+        </is>
+      </c>
+      <c r="D135" s="9" t="inlineStr">
+        <is>
+          <t>Referral to Low Vision Services for Glaucoma Patients: Referral Patterns and Characteristics of Those Who Refer.</t>
+        </is>
+      </c>
+      <c r="E135" s="9" t="inlineStr">
+        <is>
+          <t>Journal of glaucoma</t>
+        </is>
+      </c>
+      <c r="F135" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="G135" s="9" t="inlineStr">
+        <is>
+          <t>PURPOSE: To identify characteristics of ophthalmologists and practices who refer glaucoma patients to low vision services (LVS). MATERIALS AND METHODS: An online survey was distributed to members of the American Glaucoma Society. The survey queried demographics of responders and their clinical practices, criteria and barriers to referral to LVS. Survey responders were categorized as high referrers if they reported referring &gt;5 patients to LVS and low referrers if they referred ≤5. χ and Fischer exact tests were used to compare characteristics between high and low referrers. Logistic regression analyses were used to calculate odds ratios and 95% confidence intervals and determine factors associated with referrer status. RESULTS: High referrers to LVS tended to have &gt;10 patients per month who had already seen a low vision provider (53% vs. 10%, P&lt;0.001), reported following the American Academy of Ophthalmology's Preferred Practice Pattern (PPP) recommendations for LVS referrals (38% vs. 18%, P=0.011), and expressed satisfaction with their current referral practices (86% vs. 70%, P=0.049). In the fully adjusted model those who followed PPP were 2.5 times more likely to report being a high referrer as compared with a low referrer (95% confidence interval, 1.1-5.3). However, only 22% of ophthalmologists reported following these guidelines in their practice. The number of years in practice, practice location or type, volume of patients seen each week, and distance to a low vision clinic were not associated with referral. CONCLUSIONS: Familiarity with PPP guidelines may positively influence LVS referral practices.</t>
+        </is>
+      </c>
+      <c r="H135" s="11"/>
+      <c r="I135" s="11"/>
+      <c r="J135" s="11"/>
+      <c r="K135" s="11"/>
+      <c r="L135" s="11"/>
+      <c r="M135" s="9"/>
+      <c r="N135" s="12"/>
+      <c r="O135" s="12"/>
+      <c r="P135" s="12"/>
+      <c r="Q135" s="12"/>
+      <c r="R135" s="12"/>
+      <c r="S135" s="12"/>
+    </row>
+    <row r="136" spans="1:19" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A136" s="9">
+        <v>135</v>
+      </c>
+      <c r="B136" s="9">
+        <v>2023</v>
+      </c>
+      <c r="C136" s="9" t="inlineStr">
+        <is>
+          <t>Jackson, Mary Lou et al.</t>
+        </is>
+      </c>
+      <c r="D136" s="9" t="inlineStr">
+        <is>
+          <t>Vision Rehabilitation Preferred Practice Pattern®.</t>
+        </is>
+      </c>
+      <c r="E136" s="9" t="inlineStr">
+        <is>
+          <t>Ophthalmology</t>
+        </is>
+      </c>
+      <c r="F136" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="G136" s="9" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="H136" s="11"/>
+      <c r="I136" s="11"/>
+      <c r="J136" s="11"/>
+      <c r="K136" s="11"/>
+      <c r="L136" s="11"/>
+      <c r="M136" s="9"/>
+      <c r="N136" s="12"/>
+      <c r="O136" s="12"/>
+      <c r="P136" s="12"/>
+      <c r="Q136" s="12"/>
+      <c r="R136" s="12"/>
+      <c r="S136" s="12"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S128" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
-  <conditionalFormatting sqref="H2:H128">
+  <autoFilter ref="A1:S136" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <conditionalFormatting sqref="H2:H136">
     <cfRule type="expression" dxfId="8" priority="2">
       <formula>H2="Include"</formula>
     </cfRule>
@@ -10208,7 +10552,7 @@
       <formula>H2="Maybe"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J128">
+  <conditionalFormatting sqref="J2:J136">
     <cfRule type="expression" dxfId="5" priority="5">
       <formula>J2="Include"</formula>
     </cfRule>
@@ -10219,7 +10563,7 @@
       <formula>J2="Maybe"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N2:N128">
+  <conditionalFormatting sqref="N2:N136">
     <cfRule type="expression" dxfId="2" priority="8">
       <formula>N2="Include"</formula>
     </cfRule>
@@ -10230,7 +10574,7 @@
       <formula>N2="Maybe"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q2:Q128">
+  <conditionalFormatting sqref="Q2:Q136">
     <cfRule type="expression" dxfId="2" priority="11">
       <formula>Q2="Include"</formula>
     </cfRule>
@@ -10362,6 +10706,13 @@
     <hyperlink ref="F125" r:id="rId118" xr:uid="{00000000-0004-0000-0100-000075000000}"/>
     <hyperlink ref="F126" r:id="rId119" xr:uid="{00000000-0004-0000-0100-000076000000}"/>
     <hyperlink ref="F127" r:id="rId120" xr:uid="{00000000-0004-0000-0100-000077000000}"/>
+    <hyperlink ref="F129" r:id="rId121"/>
+    <hyperlink ref="F130" r:id="rId122"/>
+    <hyperlink ref="F131" r:id="rId123"/>
+    <hyperlink ref="F132" r:id="rId124"/>
+    <hyperlink ref="F134" r:id="rId125"/>
+    <hyperlink ref="F135" r:id="rId126"/>
+    <hyperlink ref="F136" r:id="rId127"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -10375,7 +10726,7 @@
           <x14:formula2>
             <xm:f>0</xm:f>
           </x14:formula2>
-          <xm:sqref>H2:H128</xm:sqref>
+          <xm:sqref>H2:H136</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0100-000001000000}">
           <x14:formula1>
@@ -10384,7 +10735,7 @@
           <x14:formula2>
             <xm:f>0</xm:f>
           </x14:formula2>
-          <xm:sqref>I2:I128 K2:K128</xm:sqref>
+          <xm:sqref>I2:I136 K2:K136</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0100-000002000000}">
           <x14:formula1>
@@ -10393,7 +10744,7 @@
           <x14:formula2>
             <xm:f>0</xm:f>
           </x14:formula2>
-          <xm:sqref>J2:J128</xm:sqref>
+          <xm:sqref>J2:J136</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -10403,7 +10754,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A2:C31"/>
+  <dimension ref="A2:C32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -10439,252 +10790,267 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="15" t="s">
-        <v>775</v>
-      </c>
-      <c r="B5" s="18">
-        <f>B3+B4</f>
-        <v>166</v>
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>Records identified – other sources</t>
+        </is>
+      </c>
+      <c r="B5" s="16">
+        <v>8</v>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>Source: key sources in the study outline, added by hand (13 Oct 2026)</t>
+        </is>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="15" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="B6" s="18">
-        <f>B5-B7</f>
-        <v>39</v>
+        <f>B3+B4+B5</f>
+        <v>174</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="15" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="B7" s="18">
-        <f>COUNTA(Screening!$D$2:$D$128)</f>
-        <v>127</v>
+        <f>B6-B8</f>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="15" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="B8" s="18">
-        <f>COUNTA(Screening!$H$2:$H$128)</f>
-        <v>40</v>
+        <f>COUNTA(Screening!$D$2:$D$136)</f>
+        <v>135</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="15" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="B9" s="18">
-        <f>COUNTIF(Screening!$H$2:$H$128,"Exclude")</f>
-        <v>27</v>
+        <f>COUNTA(Screening!$H$2:$H$136)</f>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="15" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="B10" s="18">
-        <f>COUNTIF(Screening!$H$2:$H$128,"Include")+COUNTIF(Screening!$H$2:$H$128,"Maybe")</f>
-        <v>13</v>
+        <f>COUNTIF(Screening!$H$2:$H$136,"Exclude")</f>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="15" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="B11" s="18">
-        <f>COUNTA(Screening!$J$2:$J$128)</f>
-        <v>0</v>
+        <f>COUNTIF(Screening!$H$2:$H$136,"Include")+COUNTIF(Screening!$H$2:$H$136,"Maybe")</f>
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="15" t="s">
+        <v>781</v>
+      </c>
+      <c r="B12" s="18">
+        <f>COUNTA(Screening!$J$2:$J$136)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="15" t="s">
         <v>782</v>
       </c>
-      <c r="B12" s="18">
-        <f>COUNTIF(Screening!$J$2:$J$128,"Exclude")</f>
+      <c r="B13" s="18">
+        <f>COUNTIF(Screening!$J$2:$J$136,"Exclude")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" s="19" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" s="19" t="s">
         <v>783</v>
       </c>
-      <c r="B13" s="20">
-        <f>COUNTIF(Screening!$J$2:$J$128,"Include")</f>
+      <c r="B14" s="20">
+        <f>COUNTIF(Screening!$J$2:$J$136,"Include")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="14" t="s">
+    <row r="17" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="14" t="s">
         <v>784</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" s="19" t="s">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="B18" s="19" t="s">
         <v>785</v>
       </c>
-      <c r="C17" s="19" t="s">
+      <c r="C18" s="19" t="s">
         <v>786</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="B18" s="15">
-        <f>COUNTIF(Screening!$I$2:$I$128,A18)</f>
-        <v>2</v>
-      </c>
-      <c r="C18" s="15">
-        <f>COUNTIF(Screening!$K$2:$K$128,A18)</f>
-        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="15" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="B19" s="15">
-        <f>COUNTIF(Screening!$I$2:$I$128,A19)</f>
-        <v>18</v>
+        <f>COUNTIF(Screening!$I$2:$I$136,A19)</f>
+        <v>2</v>
       </c>
       <c r="C19" s="15">
-        <f>COUNTIF(Screening!$K$2:$K$128,A19)</f>
+        <f>COUNTIF(Screening!$K$2:$K$136,A19)</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="15" t="s">
-        <v>62</v>
+        <v>24</v>
       </c>
       <c r="B20" s="15">
-        <f>COUNTIF(Screening!$I$2:$I$128,A20)</f>
-        <v>0</v>
+        <f>COUNTIF(Screening!$I$2:$I$136,A20)</f>
+        <v>18</v>
       </c>
       <c r="C20" s="15">
-        <f>COUNTIF(Screening!$K$2:$K$128,A20)</f>
+        <f>COUNTIF(Screening!$K$2:$K$136,A20)</f>
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="15" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="B21" s="15">
-        <f>COUNTIF(Screening!$I$2:$I$128,A21)</f>
-        <v>1</v>
+        <f>COUNTIF(Screening!$I$2:$I$136,A21)</f>
+        <v>0</v>
       </c>
       <c r="C21" s="15">
-        <f>COUNTIF(Screening!$K$2:$K$128,A21)</f>
+        <f>COUNTIF(Screening!$K$2:$K$136,A21)</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="15" t="s">
-        <v>95</v>
+        <v>55</v>
       </c>
       <c r="B22" s="15">
-        <f>COUNTIF(Screening!$I$2:$I$128,A22)</f>
-        <v>6</v>
+        <f>COUNTIF(Screening!$I$2:$I$136,A22)</f>
+        <v>1</v>
       </c>
       <c r="C22" s="15">
-        <f>COUNTIF(Screening!$K$2:$K$128,A22)</f>
+        <f>COUNTIF(Screening!$K$2:$K$136,A22)</f>
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="15" t="s">
-        <v>69</v>
+        <v>95</v>
       </c>
       <c r="B23" s="15">
-        <f>COUNTIF(Screening!$I$2:$I$128,A23)</f>
-        <v>0</v>
+        <f>COUNTIF(Screening!$I$2:$I$136,A23)</f>
+        <v>6</v>
       </c>
       <c r="C23" s="15">
-        <f>COUNTIF(Screening!$K$2:$K$128,A23)</f>
+        <f>COUNTIF(Screening!$K$2:$K$136,A23)</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="15" t="s">
-        <v>787</v>
+        <v>69</v>
       </c>
       <c r="B24" s="15">
-        <f>COUNTIF(Screening!$I$2:$I$128,A24)</f>
+        <f>COUNTIF(Screening!$I$2:$I$136,A24)</f>
         <v>0</v>
       </c>
       <c r="C24" s="15">
-        <f>COUNTIF(Screening!$K$2:$K$128,A24)</f>
+        <f>COUNTIF(Screening!$K$2:$K$136,A24)</f>
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="15" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="B25" s="15">
-        <f>COUNTIF(Screening!$I$2:$I$128,A25)</f>
+        <f>COUNTIF(Screening!$I$2:$I$136,A25)</f>
         <v>0</v>
       </c>
       <c r="C25" s="15">
-        <f>COUNTIF(Screening!$K$2:$K$128,A25)</f>
+        <f>COUNTIF(Screening!$K$2:$K$136,A25)</f>
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="15" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="B26" s="15">
-        <f>COUNTIF(Screening!$I$2:$I$128,A26)</f>
+        <f>COUNTIF(Screening!$I$2:$I$136,A26)</f>
         <v>0</v>
       </c>
       <c r="C26" s="15">
-        <f>COUNTIF(Screening!$K$2:$K$128,A26)</f>
+        <f>COUNTIF(Screening!$K$2:$K$136,A26)</f>
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="15" t="s">
+        <v>789</v>
+      </c>
+      <c r="B27" s="15">
+        <f>COUNTIF(Screening!$I$2:$I$136,A27)</f>
+        <v>0</v>
+      </c>
+      <c r="C27" s="15">
+        <f>COUNTIF(Screening!$K$2:$K$136,A27)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" s="15" t="s">
         <v>696</v>
       </c>
-      <c r="B27" s="15">
-        <f>COUNTIF(Screening!$I$2:$I$128,A27)</f>
+      <c r="B28" s="15">
+        <f>COUNTIF(Screening!$I$2:$I$136,A28)</f>
         <v>0</v>
       </c>
-      <c r="C27" s="15">
-        <f>COUNTIF(Screening!$K$2:$K$128,A27)</f>
+      <c r="C28" s="15">
+        <f>COUNTIF(Screening!$K$2:$K$136,A28)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A29" s="21" t="s">
+    <row r="30" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A30" s="21" t="s">
         <v>790</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A30" s="22" t="s">
-        <v>791</v>
-      </c>
-      <c r="B30" s="22">
-        <f>SUMPRODUCT((Screening!$H$2:$H$128&lt;&gt;"")*(Screening!$H$2:$H$128=Screening!$N$2:$N$128))</f>
-        <v>25</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" s="22" t="s">
+        <v>791</v>
+      </c>
+      <c r="B31" s="22">
+        <f>SUMPRODUCT((Screening!$H$2:$H$136&lt;&gt;"")*(Screening!$H$2:$H$136=Screening!$N$2:$N$136))</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" s="22" t="s">
         <v>792</v>
       </c>
-      <c r="B31" s="22">
-        <f>SUMPRODUCT((Screening!$H$2:$H$128&lt;&gt;"")*(Screening!$H$2:$H$128&lt;&gt;Screening!$N$2:$N$128))</f>
+      <c r="B32" s="22">
+        <f>SUMPRODUCT((Screening!$H$2:$H$136&lt;&gt;"")*(Screening!$H$2:$H$136&lt;&gt;Screening!$N$2:$N$136))</f>
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Snapshot of main working tree: steps 3-7 outputs synced from worktrees, workbook with AI columns for IDs 128-135, plan-doc status sections (provisional)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/LVR_screening_sheet_2.xlsx
+++ b/data/LVR_screening_sheet_2.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1264" uniqueCount="796">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1272" uniqueCount="796">
   <si>
     <t>LVR Screening Questionnaires – Title/Abstract &amp; Full-Text Screening</t>
   </si>
@@ -10231,9 +10231,17 @@
       <c r="K129" s="11"/>
       <c r="L129" s="11"/>
       <c r="M129" s="9"/>
-      <c r="N129" s="12"/>
+      <c r="N129" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
       <c r="O129" s="12"/>
-      <c r="P129" s="12"/>
+      <c r="P129" s="12" t="inlineStr">
+        <is>
+          <t>100-item yes/no everyday-object vision survey (IRT); 385 adults with VI; compared with measured logMAR VA (r=-0.72, prediction error); accuracy evaluated.</t>
+        </is>
+      </c>
       <c r="Q129" s="12"/>
       <c r="R129" s="12"/>
       <c r="S129" s="12"/>
@@ -10274,9 +10282,17 @@
       <c r="K130" s="11"/>
       <c r="L130" s="11"/>
       <c r="M130" s="9"/>
-      <c r="N130" s="12"/>
+      <c r="N130" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
       <c r="O130" s="12"/>
-      <c r="P130" s="12"/>
+      <c r="P130" s="12" t="inlineStr">
+        <is>
+          <t>Systematic review of glaucoma PROMs (GQL, GSS, NEI VFQ-25) in adults; COSMIN assessment of measurement properties, so glaucoma PROM evidence qualifies.</t>
+        </is>
+      </c>
       <c r="Q130" s="12"/>
       <c r="R130" s="12"/>
       <c r="S130" s="12"/>
@@ -10317,9 +10333,21 @@
       <c r="K131" s="11"/>
       <c r="L131" s="11"/>
       <c r="M131" s="9"/>
-      <c r="N131" s="12"/>
-      <c r="O131" s="12"/>
-      <c r="P131" s="12"/>
+      <c r="N131" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="O131" s="12" t="inlineStr">
+        <is>
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="P131" s="12" t="inlineStr">
+        <is>
+          <t>No instrument named; adults with severe glaucoma; retrospective chart review of LVR referral rates and VA/VF predictors, no self-report questionnaire evaluated.</t>
+        </is>
+      </c>
       <c r="Q131" s="12"/>
       <c r="R131" s="12"/>
       <c r="S131" s="12"/>
@@ -10360,9 +10388,21 @@
       <c r="K132" s="11"/>
       <c r="L132" s="11"/>
       <c r="M132" s="9"/>
-      <c r="N132" s="12"/>
-      <c r="O132" s="12"/>
-      <c r="P132" s="12"/>
+      <c r="N132" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="O132" s="12" t="inlineStr">
+        <is>
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="P132" s="12" t="inlineStr">
+        <is>
+          <t>MNRead, IRest and Brief Test of Attention are performance tests; adults with glaucoma; no self-report vision instrument involved or evaluated.</t>
+        </is>
+      </c>
       <c r="Q132" s="12"/>
       <c r="R132" s="12"/>
       <c r="S132" s="12"/>
@@ -10403,9 +10443,17 @@
       <c r="K133" s="11"/>
       <c r="L133" s="11"/>
       <c r="M133" s="9"/>
-      <c r="N133" s="12"/>
+      <c r="N133" s="12" t="inlineStr">
+        <is>
+          <t>Maybe</t>
+        </is>
+      </c>
       <c r="O133" s="12"/>
-      <c r="P133" s="12"/>
+      <c r="P133" s="12" t="inlineStr">
+        <is>
+          <t>No abstract; title "Legal blindness" names no instrument or population; relevance to a self-report vision questionnaire cannot be judged without full text.</t>
+        </is>
+      </c>
       <c r="Q133" s="12"/>
       <c r="R133" s="12"/>
       <c r="S133" s="12"/>
@@ -10446,9 +10494,17 @@
       <c r="K134" s="11"/>
       <c r="L134" s="11"/>
       <c r="M134" s="9"/>
-      <c r="N134" s="12"/>
+      <c r="N134" s="12" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
       <c r="O134" s="12"/>
-      <c r="P134" s="12"/>
+      <c r="P134" s="12" t="inlineStr">
+        <is>
+          <t>10-item self-rated reading difficulty questionnaire, Rasch-analysed; adults with glaucoma vs suspects; scores compared with visual field and contrast sensitivity.</t>
+        </is>
+      </c>
       <c r="Q134" s="12"/>
       <c r="R134" s="12"/>
       <c r="S134" s="12"/>
@@ -10489,9 +10545,21 @@
       <c r="K135" s="11"/>
       <c r="L135" s="11"/>
       <c r="M135" s="9"/>
-      <c r="N135" s="12"/>
-      <c r="O135" s="12"/>
-      <c r="P135" s="12"/>
+      <c r="N135" s="12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="O135" s="12" t="inlineStr">
+        <is>
+          <t>No questionnaire/screening item</t>
+        </is>
+      </c>
+      <c r="P135" s="12" t="inlineStr">
+        <is>
+          <t>No patient vision instrument; survey of American Glaucoma Society ophthalmologists on LVS referral habits; evaluates referrer characteristics and guideline adherence, not any questionnaire or screening item.</t>
+        </is>
+      </c>
       <c r="Q135" s="12"/>
       <c r="R135" s="12"/>
       <c r="S135" s="12"/>
@@ -10532,9 +10600,17 @@
       <c r="K136" s="11"/>
       <c r="L136" s="11"/>
       <c r="M136" s="9"/>
-      <c r="N136" s="12"/>
+      <c r="N136" s="12" t="inlineStr">
+        <is>
+          <t>Maybe</t>
+        </is>
+      </c>
       <c r="O136" s="12"/>
-      <c r="P136" s="12"/>
+      <c r="P136" s="12" t="inlineStr">
+        <is>
+          <t>No abstract. AAO vision rehabilitation clinical guideline; adult LVR population likely; unclear whether questionnaires or referral screening are covered or evaluated.</t>
+        </is>
+      </c>
       <c r="Q136" s="12"/>
       <c r="R136" s="12"/>
       <c r="S136" s="12"/>

</xml_diff>